<commit_message>
Fix some citations and significant digits.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/SystemValidationData.xlsx
+++ b/data/human/adult/validation/SystemValidationData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\release_updates\source\data\human\adult\validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD91FF9-D35E-4770-8A0B-544E7A81E593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4EB14ED-C40F-47BF-B9AC-E54B52784344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16620" yWindow="4695" windowWidth="28095" windowHeight="24255" tabRatio="500" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27825" yWindow="7020" windowWidth="24735" windowHeight="19980" tabRatio="500" firstSheet="4" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6596" uniqueCount="1192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6596" uniqueCount="1193">
   <si>
     <t>Patient Inputs</t>
   </si>
@@ -3289,9 +3289,6 @@
  7.0</t>
   </si>
   <si>
-    <t>guyton2006medical,         Rodgers2005physiologically</t>
-  </si>
-  <si>
     <t>p384</t>
   </si>
   <si>
@@ -3748,6 +3745,12 @@
   </si>
   <si>
     <t>TotalKidneySmallVasculature = TotalKidney/2 &lt;br&gt; SmallVasculature = TotalKidneySmallVasculature/5</t>
+  </si>
+  <si>
+    <t>[6.0,7.4]</t>
+  </si>
+  <si>
+    <t>guyton2006medical, rodgers2005physiologically</t>
   </si>
 </sst>
 </file>
@@ -5406,7 +5409,7 @@
     </row>
     <row r="12" spans="1:16">
       <c r="A12" s="10" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>844</v>
@@ -5484,7 +5487,7 @@
     </row>
     <row r="14" spans="1:16">
       <c r="A14" s="10" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>876</v>
@@ -5782,7 +5785,7 @@
     </row>
     <row r="22" spans="1:16">
       <c r="A22" s="10" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>876</v>
@@ -6020,7 +6023,7 @@
     </row>
     <row r="28" spans="1:16">
       <c r="A28" s="10" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="B28" s="18" t="s">
         <v>844</v>
@@ -6432,7 +6435,7 @@
     </row>
     <row r="39" spans="1:16" ht="96">
       <c r="A39" s="10" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B39" s="17" t="s">
         <v>862</v>
@@ -6474,7 +6477,7 @@
     </row>
     <row r="40" spans="1:16">
       <c r="A40" s="10" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="B40" s="17" t="s">
         <v>919</v>
@@ -6539,7 +6542,7 @@
         <v>49</v>
       </c>
       <c r="J41" s="26" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="L41" s="56"/>
       <c r="M41" s="66" t="s">
@@ -6964,7 +6967,7 @@
     </row>
     <row r="53" spans="1:16" ht="108">
       <c r="A53" s="10" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="B53" s="26" t="s">
         <v>844</v>
@@ -9400,20 +9403,20 @@
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
       <c r="F5" s="8" t="s">
-        <v>1039</v>
+        <v>1191</v>
       </c>
       <c r="G5" s="8" t="s">
+        <v>1192</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>1040</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>1041</v>
       </c>
       <c r="I5" s="14" t="s">
         <v>49</v>
       </c>
       <c r="J5" s="109"/>
       <c r="K5" s="8" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>1039</v>
@@ -9433,7 +9436,7 @@
     </row>
     <row r="6" spans="1:16" s="1" customFormat="1">
       <c r="A6" s="10" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>17</v>
@@ -9455,7 +9458,7 @@
         <v>49</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="K6" s="8"/>
       <c r="L6" s="8">
@@ -9474,7 +9477,7 @@
     </row>
     <row r="7" spans="1:16">
       <c r="A7" s="67" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>14</v>
@@ -9512,7 +9515,7 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" s="67" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="8" t="s">
@@ -9524,10 +9527,10 @@
         <v>0.85</v>
       </c>
       <c r="G8" s="111" t="s">
+        <v>1046</v>
+      </c>
+      <c r="H8" s="111" t="s">
         <v>1047</v>
-      </c>
-      <c r="H8" s="111" t="s">
-        <v>1048</v>
       </c>
       <c r="I8" s="14" t="s">
         <v>49</v>
@@ -9552,7 +9555,7 @@
     </row>
     <row r="9" spans="1:16">
       <c r="A9" s="120" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>923</v>
@@ -9590,7 +9593,7 @@
     </row>
     <row r="10" spans="1:16" s="1" customFormat="1" ht="26.25" customHeight="1">
       <c r="A10" s="28" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>1</v>
@@ -9640,7 +9643,7 @@
     </row>
     <row r="11" spans="1:16">
       <c r="A11" s="67" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>14</v>
@@ -9657,7 +9660,7 @@
         <v>104</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="I11" s="14" t="s">
         <v>49</v>
@@ -9682,7 +9685,7 @@
     </row>
     <row r="12" spans="1:16" s="1" customFormat="1">
       <c r="A12" s="67" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>14</v>
@@ -9699,7 +9702,7 @@
         <v>104</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>49</v>
@@ -9724,7 +9727,7 @@
     </row>
     <row r="13" spans="1:16" s="1" customFormat="1" ht="26.25" customHeight="1">
       <c r="A13" s="28" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>1</v>
@@ -9774,7 +9777,7 @@
     </row>
     <row r="14" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A14" s="30" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>923</v>
@@ -9796,32 +9799,32 @@
         <v>273</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I14" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J14" s="17"/>
       <c r="K14" s="33" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="L14" s="5">
         <v>3140</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N14" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O14" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P14" s="14"/>
     </row>
     <row r="15" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A15" s="30" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>17</v>
@@ -9839,20 +9842,20 @@
         <v>1032</v>
       </c>
       <c r="H15" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I15" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J15" s="17"/>
       <c r="K15" s="33" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="L15" s="5">
         <v>3140</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N15" s="5" t="s">
         <v>71</v>
@@ -9864,7 +9867,7 @@
     </row>
     <row r="16" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A16" s="30" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>17</v>
@@ -9882,20 +9885,20 @@
         <v>1032</v>
       </c>
       <c r="H16" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I16" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J16" s="17"/>
       <c r="K16" s="33" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="L16" s="5">
         <v>3140</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N16" s="5" t="s">
         <v>71</v>
@@ -9907,7 +9910,7 @@
     </row>
     <row r="17" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A17" s="30" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>923</v>
@@ -9929,32 +9932,32 @@
         <v>273</v>
       </c>
       <c r="H17" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I17" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J17" s="17"/>
       <c r="K17" s="33" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="L17" s="5">
         <v>2680</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N17" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O17" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P17" s="14"/>
     </row>
     <row r="18" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A18" s="30" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>17</v>
@@ -9972,20 +9975,20 @@
         <v>1032</v>
       </c>
       <c r="H18" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I18" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J18" s="17"/>
       <c r="K18" s="33" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="L18" s="5">
         <v>2680</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N18" s="5" t="s">
         <v>71</v>
@@ -9997,7 +10000,7 @@
     </row>
     <row r="19" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A19" s="30" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>17</v>
@@ -10015,20 +10018,20 @@
         <v>1032</v>
       </c>
       <c r="H19" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I19" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J19" s="17"/>
       <c r="K19" s="33" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="L19" s="5">
         <v>2680</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N19" s="5" t="s">
         <v>71</v>
@@ -10040,7 +10043,7 @@
     </row>
     <row r="20" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A20" s="30" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>923</v>
@@ -10062,32 +10065,32 @@
         <v>273</v>
       </c>
       <c r="H20" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I20" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J20" s="17"/>
       <c r="K20" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L20" s="5">
         <v>1020</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N20" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O20" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P20" s="14"/>
     </row>
     <row r="21" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A21" s="30" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>17</v>
@@ -10105,20 +10108,20 @@
         <v>1032</v>
       </c>
       <c r="H21" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I21" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J21" s="17"/>
       <c r="K21" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L21" s="5">
         <v>1020</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N21" s="5" t="s">
         <v>71</v>
@@ -10130,7 +10133,7 @@
     </row>
     <row r="22" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A22" s="30" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>17</v>
@@ -10148,20 +10151,20 @@
         <v>1032</v>
       </c>
       <c r="H22" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I22" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J22" s="17"/>
       <c r="K22" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L22" s="5">
         <v>1020</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N22" s="5" t="s">
         <v>71</v>
@@ -10173,7 +10176,7 @@
     </row>
     <row r="23" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A23" s="30" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>923</v>
@@ -10195,32 +10198,32 @@
         <v>273</v>
       </c>
       <c r="H23" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I23" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J23" s="17"/>
       <c r="K23" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L23" s="5">
         <v>730</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N23" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O23" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P23" s="14"/>
     </row>
     <row r="24" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A24" s="30" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>17</v>
@@ -10238,20 +10241,20 @@
         <v>1032</v>
       </c>
       <c r="H24" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I24" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J24" s="17"/>
       <c r="K24" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L24" s="5">
         <v>730</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N24" s="5" t="s">
         <v>71</v>
@@ -10263,7 +10266,7 @@
     </row>
     <row r="25" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A25" s="30" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>17</v>
@@ -10281,20 +10284,20 @@
         <v>1032</v>
       </c>
       <c r="H25" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I25" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J25" s="17"/>
       <c r="K25" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L25" s="5">
         <v>730</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N25" s="5" t="s">
         <v>71</v>
@@ -10306,7 +10309,7 @@
     </row>
     <row r="26" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A26" s="30" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>923</v>
@@ -10328,32 +10331,32 @@
         <v>273</v>
       </c>
       <c r="H26" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I26" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J26" s="17"/>
       <c r="K26" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L26" s="5">
         <v>110</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N26" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O26" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P26" s="14"/>
     </row>
     <row r="27" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A27" s="30" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>17</v>
@@ -10371,20 +10374,20 @@
         <v>1032</v>
       </c>
       <c r="H27" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I27" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J27" s="17"/>
       <c r="K27" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L27" s="5">
         <v>110</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N27" s="5" t="s">
         <v>71</v>
@@ -10396,7 +10399,7 @@
     </row>
     <row r="28" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A28" s="30" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>17</v>
@@ -10414,20 +10417,20 @@
         <v>1032</v>
       </c>
       <c r="H28" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I28" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J28" s="17"/>
       <c r="K28" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L28" s="5">
         <v>110</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N28" s="5" t="s">
         <v>71</v>
@@ -10439,7 +10442,7 @@
     </row>
     <row r="29" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A29" s="30" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>923</v>
@@ -10461,32 +10464,32 @@
         <v>273</v>
       </c>
       <c r="H29" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I29" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J29" s="17"/>
       <c r="K29" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L29" s="5">
         <v>110</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N29" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O29" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P29" s="14"/>
     </row>
     <row r="30" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A30" s="30" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>17</v>
@@ -10504,20 +10507,20 @@
         <v>1032</v>
       </c>
       <c r="H30" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I30" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J30" s="17"/>
       <c r="K30" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L30" s="5">
         <v>110</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N30" s="5" t="s">
         <v>71</v>
@@ -10529,7 +10532,7 @@
     </row>
     <row r="31" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A31" s="30" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>17</v>
@@ -10547,20 +10550,20 @@
         <v>1032</v>
       </c>
       <c r="H31" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I31" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J31" s="17"/>
       <c r="K31" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L31" s="5">
         <v>110</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N31" s="5" t="s">
         <v>71</v>
@@ -10572,7 +10575,7 @@
     </row>
     <row r="32" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A32" s="30" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>923</v>
@@ -10594,32 +10597,32 @@
         <v>273</v>
       </c>
       <c r="H32" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I32" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J32" s="17"/>
       <c r="K32" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L32" s="5">
         <v>1030</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N32" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O32" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P32" s="14"/>
     </row>
     <row r="33" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A33" s="30" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>17</v>
@@ -10637,20 +10640,20 @@
         <v>1032</v>
       </c>
       <c r="H33" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I33" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J33" s="17"/>
       <c r="K33" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L33" s="5">
         <v>1030</v>
       </c>
       <c r="M33" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N33" s="5" t="s">
         <v>71</v>
@@ -10662,7 +10665,7 @@
     </row>
     <row r="34" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A34" s="30" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>17</v>
@@ -10680,20 +10683,20 @@
         <v>1032</v>
       </c>
       <c r="H34" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I34" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J34" s="17"/>
       <c r="K34" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L34" s="5">
         <v>1030</v>
       </c>
       <c r="M34" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N34" s="5" t="s">
         <v>71</v>
@@ -10705,7 +10708,7 @@
     </row>
     <row r="35" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A35" s="30" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>923</v>
@@ -10729,32 +10732,32 @@
         <v>273</v>
       </c>
       <c r="H35" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I35" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J35" s="17"/>
       <c r="K35" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L35" s="5">
         <v>160</v>
       </c>
       <c r="M35" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N35" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O35" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P35" s="14"/>
     </row>
     <row r="36" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A36" s="30" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>17</v>
@@ -10772,20 +10775,20 @@
         <v>1032</v>
       </c>
       <c r="H36" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I36" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J36" s="17"/>
       <c r="K36" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L36" s="5">
         <v>160</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N36" s="5" t="s">
         <v>71</v>
@@ -10797,7 +10800,7 @@
     </row>
     <row r="37" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A37" s="30" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>17</v>
@@ -10815,20 +10818,20 @@
         <v>1032</v>
       </c>
       <c r="H37" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I37" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J37" s="17"/>
       <c r="K37" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L37" s="5">
         <v>160</v>
       </c>
       <c r="M37" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N37" s="5" t="s">
         <v>71</v>
@@ -10840,7 +10843,7 @@
     </row>
     <row r="38" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A38" s="30" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>923</v>
@@ -10864,32 +10867,32 @@
         <v>273</v>
       </c>
       <c r="H38" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I38" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J38" s="17"/>
       <c r="K38" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L38" s="5">
         <v>160</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N38" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O38" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P38" s="14"/>
     </row>
     <row r="39" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A39" s="30" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>17</v>
@@ -10907,20 +10910,20 @@
         <v>1032</v>
       </c>
       <c r="H39" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I39" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J39" s="17"/>
       <c r="K39" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L39" s="5">
         <v>160</v>
       </c>
       <c r="M39" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N39" s="5" t="s">
         <v>71</v>
@@ -10932,7 +10935,7 @@
     </row>
     <row r="40" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A40" s="30" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>17</v>
@@ -10950,20 +10953,20 @@
         <v>1032</v>
       </c>
       <c r="H40" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I40" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J40" s="17"/>
       <c r="K40" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L40" s="5">
         <v>160</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N40" s="5" t="s">
         <v>71</v>
@@ -10975,7 +10978,7 @@
     </row>
     <row r="41" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A41" s="30" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>923</v>
@@ -10997,32 +11000,32 @@
         <v>273</v>
       </c>
       <c r="H41" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I41" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J41" s="17"/>
       <c r="K41" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L41" s="5">
         <v>13090</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N41" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O41" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P41" s="14"/>
     </row>
     <row r="42" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A42" s="30" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>17</v>
@@ -11040,20 +11043,20 @@
         <v>1032</v>
       </c>
       <c r="H42" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I42" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J42" s="17"/>
       <c r="K42" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L42" s="5">
         <v>13090</v>
       </c>
       <c r="M42" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N42" s="5" t="s">
         <v>71</v>
@@ -11065,7 +11068,7 @@
     </row>
     <row r="43" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A43" s="30" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>17</v>
@@ -11083,20 +11086,20 @@
         <v>1032</v>
       </c>
       <c r="H43" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I43" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J43" s="17"/>
       <c r="K43" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L43" s="5">
         <v>13090</v>
       </c>
       <c r="M43" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N43" s="5" t="s">
         <v>71</v>
@@ -11108,7 +11111,7 @@
     </row>
     <row r="44" spans="1:16">
       <c r="A44" s="30" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="B44" s="18" t="s">
         <v>89</v>
@@ -11119,10 +11122,10 @@
       <c r="D44" s="14"/>
       <c r="E44" s="14"/>
       <c r="F44" s="52" t="s">
+        <v>1090</v>
+      </c>
+      <c r="G44" s="17" t="s">
         <v>1091</v>
-      </c>
-      <c r="G44" s="17" t="s">
-        <v>1092</v>
       </c>
       <c r="H44" s="17"/>
       <c r="I44" s="26" t="s">
@@ -11132,7 +11135,7 @@
       <c r="K44" s="33"/>
       <c r="L44" s="21"/>
       <c r="M44" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N44" s="5" t="s">
         <v>71</v>
@@ -11144,7 +11147,7 @@
     </row>
     <row r="45" spans="1:16">
       <c r="A45" s="30" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="B45" s="18" t="s">
         <v>89</v>
@@ -11155,7 +11158,7 @@
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
       <c r="F45" s="113" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="G45" s="17" t="s">
         <v>547</v>
@@ -11166,11 +11169,11 @@
       </c>
       <c r="J45" s="5"/>
       <c r="K45" s="33" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="L45" s="4"/>
       <c r="M45" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N45" s="5" t="s">
         <v>71</v>
@@ -11182,7 +11185,7 @@
     </row>
     <row r="46" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A46" s="30" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>923</v>
@@ -11204,32 +11207,32 @@
         <v>273</v>
       </c>
       <c r="H46" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I46" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J46" s="17"/>
       <c r="K46" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L46" s="5">
         <v>190</v>
       </c>
       <c r="M46" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N46" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O46" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P46" s="14"/>
     </row>
     <row r="47" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A47" s="30" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>17</v>
@@ -11247,20 +11250,20 @@
         <v>1032</v>
       </c>
       <c r="H47" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I47" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J47" s="17"/>
       <c r="K47" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L47" s="5">
         <v>190</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N47" s="5" t="s">
         <v>71</v>
@@ -11272,7 +11275,7 @@
     </row>
     <row r="48" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A48" s="30" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>17</v>
@@ -11290,20 +11293,20 @@
         <v>1032</v>
       </c>
       <c r="H48" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I48" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J48" s="17"/>
       <c r="K48" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L48" s="5">
         <v>190</v>
       </c>
       <c r="M48" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N48" s="5" t="s">
         <v>71</v>
@@ -11315,7 +11318,7 @@
     </row>
     <row r="49" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A49" s="30" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>923</v>
@@ -11337,32 +11340,32 @@
         <v>273</v>
       </c>
       <c r="H49" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I49" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J49" s="17"/>
       <c r="K49" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L49" s="5">
         <v>1550</v>
       </c>
       <c r="M49" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N49" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O49" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P49" s="14"/>
     </row>
     <row r="50" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A50" s="30" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>17</v>
@@ -11380,20 +11383,20 @@
         <v>1032</v>
       </c>
       <c r="H50" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I50" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J50" s="17"/>
       <c r="K50" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L50" s="5">
         <v>1550</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N50" s="5" t="s">
         <v>71</v>
@@ -11405,7 +11408,7 @@
     </row>
     <row r="51" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A51" s="30" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>17</v>
@@ -11423,20 +11426,20 @@
         <v>1032</v>
       </c>
       <c r="H51" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I51" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J51" s="17"/>
       <c r="K51" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L51" s="5">
         <v>1550</v>
       </c>
       <c r="M51" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N51" s="5" t="s">
         <v>71</v>
@@ -11448,7 +11451,7 @@
     </row>
     <row r="52" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A52" s="30" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>923</v>
@@ -11470,32 +11473,32 @@
         <v>273</v>
       </c>
       <c r="H52" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I52" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J52" s="17"/>
       <c r="K52" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L52" s="5">
         <v>100</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N52" s="5" t="s">
         <v>51</v>
       </c>
       <c r="O52" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P52" s="14"/>
     </row>
     <row r="53" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A53" s="30" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>17</v>
@@ -11513,20 +11516,20 @@
         <v>1032</v>
       </c>
       <c r="H53" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I53" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J53" s="17"/>
       <c r="K53" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L53" s="5">
         <v>100</v>
       </c>
       <c r="M53" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N53" s="5" t="s">
         <v>71</v>
@@ -11538,7 +11541,7 @@
     </row>
     <row r="54" spans="1:16" s="1" customFormat="1" ht="12">
       <c r="A54" s="30" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>17</v>
@@ -11556,20 +11559,20 @@
         <v>1032</v>
       </c>
       <c r="H54" s="26" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="I54" s="26" t="s">
         <v>49</v>
       </c>
       <c r="J54" s="17"/>
       <c r="K54" s="33" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="L54" s="5">
         <v>100</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="N54" s="5" t="s">
         <v>71</v>
@@ -11581,7 +11584,7 @@
     </row>
     <row r="55" spans="1:16" ht="24">
       <c r="A55" s="28" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>1</v>
@@ -11631,7 +11634,7 @@
     </row>
     <row r="56" spans="1:16" ht="24.75">
       <c r="A56" s="30" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="B56" s="18" t="s">
         <v>89</v>
@@ -11642,7 +11645,7 @@
       <c r="D56" s="14"/>
       <c r="E56" s="14"/>
       <c r="F56" s="18" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="G56" s="18" t="s">
         <v>143</v>
@@ -11653,23 +11656,23 @@
       </c>
       <c r="J56" s="18"/>
       <c r="K56" s="114" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="L56" s="14"/>
       <c r="M56" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N56" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O56" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P56" s="14"/>
     </row>
     <row r="57" spans="1:16">
       <c r="A57" s="30" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B57" s="18" t="s">
         <v>89</v>
@@ -11693,19 +11696,19 @@
         <v>1034</v>
       </c>
       <c r="M57" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N57" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O57" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P57" s="14"/>
     </row>
     <row r="58" spans="1:16">
       <c r="A58" s="30" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="B58" s="18" t="s">
         <v>89</v>
@@ -11719,10 +11722,10 @@
         <v>25</v>
       </c>
       <c r="G58" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H58" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H58" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I58" s="18" t="s">
         <v>49</v>
@@ -11733,19 +11736,19 @@
         <v>1036</v>
       </c>
       <c r="M58" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N58" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O58" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P58" s="14"/>
     </row>
     <row r="59" spans="1:16">
       <c r="A59" s="30" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="B59" s="18" t="s">
         <v>89</v>
@@ -11759,10 +11762,10 @@
         <v>1.2</v>
       </c>
       <c r="G59" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H59" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H59" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I59" s="18" t="s">
         <v>49</v>
@@ -11770,22 +11773,22 @@
       <c r="J59" s="17"/>
       <c r="K59" s="19"/>
       <c r="L59" s="8" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="M59" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N59" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O59" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P59" s="14"/>
     </row>
     <row r="60" spans="1:16" ht="24">
       <c r="A60" s="30" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="B60" s="115" t="s">
         <v>89</v>
@@ -11796,7 +11799,7 @@
       <c r="D60" s="115"/>
       <c r="E60" s="115"/>
       <c r="F60" s="116" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="G60" s="115"/>
       <c r="H60" s="116"/>
@@ -11805,23 +11808,23 @@
       </c>
       <c r="J60" s="116"/>
       <c r="K60" s="116" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="L60" s="8"/>
       <c r="M60" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N60" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O60" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P60" s="14"/>
     </row>
     <row r="61" spans="1:16">
       <c r="A61" s="30" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="B61" s="18" t="s">
         <v>89</v>
@@ -11835,10 +11838,10 @@
         <v>116</v>
       </c>
       <c r="G61" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H61" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H61" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I61" s="18" t="s">
         <v>49</v>
@@ -11847,19 +11850,19 @@
       <c r="K61" s="33"/>
       <c r="L61" s="14"/>
       <c r="M61" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N61" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O61" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P61" s="14"/>
     </row>
     <row r="62" spans="1:16" ht="36.75">
       <c r="A62" s="30" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B62" s="115"/>
       <c r="C62" s="116"/>
@@ -11873,26 +11876,26 @@
       </c>
       <c r="J62" s="116"/>
       <c r="K62" s="117" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="L62" s="14"/>
       <c r="M62" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N62" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O62" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P62" s="14"/>
     </row>
     <row r="63" spans="1:16" ht="72.75">
       <c r="A63" s="30" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B63" s="17" t="s">
         <v>1121</v>
-      </c>
-      <c r="B63" s="17" t="s">
-        <v>1122</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>46</v>
@@ -11900,36 +11903,36 @@
       <c r="D63" s="14"/>
       <c r="E63" s="14"/>
       <c r="F63" s="8" t="s">
+        <v>1122</v>
+      </c>
+      <c r="G63" s="17" t="s">
         <v>1123</v>
       </c>
-      <c r="G63" s="17" t="s">
+      <c r="H63" s="17" t="s">
         <v>1124</v>
-      </c>
-      <c r="H63" s="17" t="s">
-        <v>1125</v>
       </c>
       <c r="I63" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J63" s="17"/>
       <c r="K63" s="114" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="L63" s="4"/>
       <c r="M63" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N63" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O63" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P63" s="14"/>
     </row>
     <row r="64" spans="1:16">
       <c r="A64" s="30" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="B64" s="18" t="s">
         <v>89</v>
@@ -11943,10 +11946,10 @@
         <v>5.9</v>
       </c>
       <c r="G64" s="17" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H64" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H64" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I64" s="18" t="s">
         <v>49</v>
@@ -11955,19 +11958,19 @@
       <c r="K64" s="33"/>
       <c r="L64" s="21"/>
       <c r="M64" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N64" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O64" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P64" s="14"/>
     </row>
     <row r="65" spans="1:16">
       <c r="A65" s="30" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="B65" s="18" t="s">
         <v>89</v>
@@ -11987,26 +11990,26 @@
       </c>
       <c r="J65" s="26"/>
       <c r="K65" s="33" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="L65" s="4"/>
       <c r="M65" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N65" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O65" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P65" s="14"/>
     </row>
     <row r="66" spans="1:16" ht="24.75">
       <c r="A66" s="30" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B66" s="26" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>46</v>
@@ -12014,36 +12017,36 @@
       <c r="D66" s="14"/>
       <c r="E66" s="14"/>
       <c r="F66" s="26" t="s">
+        <v>1130</v>
+      </c>
+      <c r="G66" s="17" t="s">
         <v>1131</v>
       </c>
-      <c r="G66" s="17" t="s">
+      <c r="H66" s="26" t="s">
         <v>1132</v>
-      </c>
-      <c r="H66" s="26" t="s">
-        <v>1133</v>
       </c>
       <c r="I66" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J66" s="5"/>
       <c r="K66" s="114" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="L66" s="4"/>
       <c r="M66" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N66" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O66" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P66" s="14"/>
     </row>
     <row r="67" spans="1:16" ht="48.75">
       <c r="A67" s="30" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="B67" s="18" t="s">
         <v>89</v>
@@ -12054,36 +12057,36 @@
       <c r="D67" s="14"/>
       <c r="E67" s="14"/>
       <c r="F67" s="26" t="s">
+        <v>1134</v>
+      </c>
+      <c r="G67" s="17" t="s">
         <v>1135</v>
       </c>
-      <c r="G67" s="17" t="s">
+      <c r="H67" s="26" t="s">
         <v>1136</v>
-      </c>
-      <c r="H67" s="26" t="s">
-        <v>1137</v>
       </c>
       <c r="I67" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J67" s="5"/>
       <c r="K67" s="33" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="L67" s="4"/>
       <c r="M67" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N67" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O67" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P67" s="14"/>
     </row>
     <row r="68" spans="1:16" ht="24">
       <c r="A68" s="30" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="B68" s="115"/>
       <c r="C68" s="116"/>
@@ -12097,26 +12100,26 @@
       </c>
       <c r="J68" s="116"/>
       <c r="K68" s="115" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="L68" s="4"/>
       <c r="M68" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N68" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O68" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P68" s="14"/>
     </row>
     <row r="69" spans="1:16">
       <c r="A69" s="30" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B69" s="18" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>46</v>
@@ -12124,13 +12127,13 @@
       <c r="D69" s="14"/>
       <c r="E69" s="14"/>
       <c r="F69" s="26" t="s">
+        <v>1141</v>
+      </c>
+      <c r="G69" s="17" t="s">
+        <v>1135</v>
+      </c>
+      <c r="H69" s="26" t="s">
         <v>1142</v>
-      </c>
-      <c r="G69" s="17" t="s">
-        <v>1136</v>
-      </c>
-      <c r="H69" s="26" t="s">
-        <v>1143</v>
       </c>
       <c r="I69" s="18" t="s">
         <v>49</v>
@@ -12139,19 +12142,19 @@
       <c r="K69" s="26"/>
       <c r="L69" s="4"/>
       <c r="M69" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N69" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O69" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P69" s="14"/>
     </row>
     <row r="70" spans="1:16" ht="24">
       <c r="A70" s="30" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="B70" s="18" t="s">
         <v>89</v>
@@ -12162,7 +12165,7 @@
       <c r="D70" s="14"/>
       <c r="E70" s="14"/>
       <c r="F70" s="8" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="G70" s="17"/>
       <c r="H70" s="8"/>
@@ -12171,23 +12174,23 @@
       </c>
       <c r="J70" s="8"/>
       <c r="K70" s="116" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="L70" s="4"/>
       <c r="M70" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N70" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O70" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P70" s="14"/>
     </row>
     <row r="71" spans="1:16">
       <c r="A71" s="10" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="B71" s="18" t="s">
         <v>89</v>
@@ -12201,10 +12204,10 @@
         <v>4.5</v>
       </c>
       <c r="G71" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H71" s="18" t="s">
         <v>1112</v>
-      </c>
-      <c r="H71" s="18" t="s">
-        <v>1113</v>
       </c>
       <c r="I71" s="18" t="s">
         <v>49</v>
@@ -12213,19 +12216,19 @@
       <c r="K71" s="33"/>
       <c r="L71" s="4"/>
       <c r="M71" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N71" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O71" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P71" s="14"/>
     </row>
     <row r="72" spans="1:16">
       <c r="A72" s="30" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="B72" s="18" t="s">
         <v>89</v>
@@ -12239,10 +12242,10 @@
         <v>145</v>
       </c>
       <c r="G72" s="17" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H72" s="26" t="s">
         <v>1112</v>
-      </c>
-      <c r="H72" s="26" t="s">
-        <v>1113</v>
       </c>
       <c r="I72" s="18" t="s">
         <v>49</v>
@@ -12251,19 +12254,19 @@
       <c r="K72" s="33"/>
       <c r="L72" s="4"/>
       <c r="M72" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N72" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O72" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P72" s="14"/>
     </row>
     <row r="73" spans="1:16">
       <c r="A73" s="30" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="B73" s="36" t="s">
         <v>89</v>
@@ -12281,23 +12284,23 @@
       </c>
       <c r="J73" s="118"/>
       <c r="K73" s="114" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="L73" s="4"/>
       <c r="M73" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N73" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O73" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P73" s="14"/>
     </row>
     <row r="74" spans="1:16" ht="36">
       <c r="A74" s="30" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="B74" s="26" t="s">
         <v>66</v>
@@ -12319,23 +12322,23 @@
       </c>
       <c r="J74" s="119"/>
       <c r="K74" s="47" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="L74" s="4"/>
       <c r="M74" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N74" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O74" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P74" s="14"/>
     </row>
     <row r="75" spans="1:16" ht="24.75">
       <c r="A75" s="30" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="B75" s="18" t="s">
         <v>89</v>
@@ -12346,7 +12349,7 @@
       <c r="D75" s="14"/>
       <c r="E75" s="14"/>
       <c r="F75" s="18" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="G75" s="18"/>
       <c r="H75" s="18"/>
@@ -12355,23 +12358,23 @@
       </c>
       <c r="J75" s="18"/>
       <c r="K75" s="114" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="L75" s="4"/>
       <c r="M75" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N75" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O75" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P75" s="14"/>
     </row>
     <row r="76" spans="1:16">
       <c r="A76" s="30" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B76" s="18" t="s">
         <v>89</v>
@@ -12391,23 +12394,23 @@
       </c>
       <c r="J76" s="8"/>
       <c r="K76" s="35" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="L76" s="4"/>
       <c r="M76" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N76" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O76" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P76" s="14"/>
     </row>
     <row r="77" spans="1:16">
       <c r="A77" s="30" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B77" s="18" t="s">
         <v>89</v>
@@ -12421,10 +12424,10 @@
         <v>16</v>
       </c>
       <c r="G77" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H77" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H77" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I77" s="18" t="s">
         <v>49</v>
@@ -12433,19 +12436,19 @@
       <c r="K77" s="19"/>
       <c r="L77" s="4"/>
       <c r="M77" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N77" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O77" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P77" s="14"/>
     </row>
     <row r="78" spans="1:16">
       <c r="A78" s="30" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B78" s="18" t="s">
         <v>89</v>
@@ -12459,10 +12462,10 @@
         <v>1E-4</v>
       </c>
       <c r="G78" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H78" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H78" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I78" s="18" t="s">
         <v>49</v>
@@ -12471,19 +12474,19 @@
       <c r="K78" s="19"/>
       <c r="L78" s="4"/>
       <c r="M78" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N78" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O78" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P78" s="14"/>
     </row>
     <row r="79" spans="1:16" ht="24">
       <c r="A79" s="30" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="B79" s="115" t="s">
         <v>89</v>
@@ -12494,7 +12497,7 @@
       <c r="D79" s="115"/>
       <c r="E79" s="115"/>
       <c r="F79" s="116" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="G79" s="115"/>
       <c r="H79" s="116"/>
@@ -12503,23 +12506,23 @@
       </c>
       <c r="J79" s="116"/>
       <c r="K79" s="116" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="L79" s="4"/>
       <c r="M79" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N79" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O79" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P79" s="14"/>
     </row>
     <row r="80" spans="1:16">
       <c r="A80" s="30" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="B80" s="18" t="s">
         <v>89</v>
@@ -12533,10 +12536,10 @@
         <v>20</v>
       </c>
       <c r="G80" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H80" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H80" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I80" s="18" t="s">
         <v>49</v>
@@ -12545,19 +12548,19 @@
       <c r="K80" s="33"/>
       <c r="L80" s="4"/>
       <c r="M80" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N80" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O80" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P80" s="14"/>
     </row>
     <row r="81" spans="1:16" ht="36.75">
       <c r="A81" s="30" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B81" s="18" t="s">
         <v>89</v>
@@ -12575,26 +12578,26 @@
       </c>
       <c r="J81" s="17"/>
       <c r="K81" s="114" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="L81" s="4"/>
       <c r="M81" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N81" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O81" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P81" s="14"/>
     </row>
     <row r="82" spans="1:16" ht="72.75">
       <c r="A82" s="30" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B82" s="17" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C82" s="8" t="s">
         <v>46</v>
@@ -12602,36 +12605,36 @@
       <c r="D82" s="14"/>
       <c r="E82" s="14"/>
       <c r="F82" s="8" t="s">
+        <v>1122</v>
+      </c>
+      <c r="G82" s="17" t="s">
         <v>1123</v>
       </c>
-      <c r="G82" s="17" t="s">
+      <c r="H82" s="17" t="s">
         <v>1124</v>
-      </c>
-      <c r="H82" s="17" t="s">
-        <v>1125</v>
       </c>
       <c r="I82" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J82" s="17"/>
       <c r="K82" s="114" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="L82" s="4"/>
       <c r="M82" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N82" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O82" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P82" s="14"/>
     </row>
     <row r="83" spans="1:16">
       <c r="A83" s="30" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B83" s="18" t="s">
         <v>89</v>
@@ -12645,10 +12648,10 @@
         <v>0</v>
       </c>
       <c r="G83" s="17" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H83" s="17" t="s">
         <v>1112</v>
-      </c>
-      <c r="H83" s="17" t="s">
-        <v>1113</v>
       </c>
       <c r="I83" s="18" t="s">
         <v>49</v>
@@ -12657,19 +12660,19 @@
       <c r="K83" s="33"/>
       <c r="L83" s="21"/>
       <c r="M83" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N83" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O83" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P83" s="14"/>
     </row>
     <row r="84" spans="1:16">
       <c r="A84" s="30" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="B84" s="18" t="s">
         <v>89</v>
@@ -12689,26 +12692,26 @@
       </c>
       <c r="J84" s="26"/>
       <c r="K84" s="33" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="L84" s="4"/>
       <c r="M84" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N84" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O84" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P84" s="14"/>
     </row>
     <row r="85" spans="1:16" ht="24.75">
       <c r="A85" s="30" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B85" s="26" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>46</v>
@@ -12716,36 +12719,36 @@
       <c r="D85" s="14"/>
       <c r="E85" s="14"/>
       <c r="F85" s="26" t="s">
+        <v>1130</v>
+      </c>
+      <c r="G85" s="17" t="s">
         <v>1131</v>
       </c>
-      <c r="G85" s="17" t="s">
+      <c r="H85" s="26" t="s">
         <v>1132</v>
-      </c>
-      <c r="H85" s="26" t="s">
-        <v>1133</v>
       </c>
       <c r="I85" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J85" s="5"/>
       <c r="K85" s="114" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="L85" s="4"/>
       <c r="M85" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N85" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O85" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P85" s="14"/>
     </row>
     <row r="86" spans="1:16" ht="48.75">
       <c r="A86" s="30" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B86" s="18" t="s">
         <v>89</v>
@@ -12756,36 +12759,36 @@
       <c r="D86" s="14"/>
       <c r="E86" s="14"/>
       <c r="F86" s="26" t="s">
+        <v>1134</v>
+      </c>
+      <c r="G86" s="17" t="s">
         <v>1135</v>
       </c>
-      <c r="G86" s="17" t="s">
+      <c r="H86" s="26" t="s">
         <v>1136</v>
-      </c>
-      <c r="H86" s="26" t="s">
-        <v>1137</v>
       </c>
       <c r="I86" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J86" s="5"/>
       <c r="K86" s="33" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="L86" s="4"/>
       <c r="M86" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N86" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O86" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P86" s="14"/>
     </row>
     <row r="87" spans="1:16">
       <c r="A87" s="30" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="B87" s="18" t="s">
         <v>89</v>
@@ -12805,22 +12808,22 @@
       <c r="K87" s="26"/>
       <c r="L87" s="4"/>
       <c r="M87" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N87" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O87" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P87" s="14"/>
     </row>
     <row r="88" spans="1:16">
       <c r="A88" s="30" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="B88" s="18" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C88" s="8" t="s">
         <v>46</v>
@@ -12828,13 +12831,13 @@
       <c r="D88" s="14"/>
       <c r="E88" s="14"/>
       <c r="F88" s="26" t="s">
+        <v>1141</v>
+      </c>
+      <c r="G88" s="17" t="s">
+        <v>1135</v>
+      </c>
+      <c r="H88" s="26" t="s">
         <v>1142</v>
-      </c>
-      <c r="G88" s="17" t="s">
-        <v>1136</v>
-      </c>
-      <c r="H88" s="26" t="s">
-        <v>1143</v>
       </c>
       <c r="I88" s="18" t="s">
         <v>49</v>
@@ -12843,19 +12846,19 @@
       <c r="K88" s="26"/>
       <c r="L88" s="4"/>
       <c r="M88" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N88" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O88" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P88" s="14"/>
     </row>
     <row r="89" spans="1:16" ht="24">
       <c r="A89" s="30" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B89" s="18" t="s">
         <v>89</v>
@@ -12866,7 +12869,7 @@
       <c r="D89" s="14"/>
       <c r="E89" s="14"/>
       <c r="F89" s="8" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="G89" s="17"/>
       <c r="H89" s="8"/>
@@ -12875,23 +12878,23 @@
       </c>
       <c r="J89" s="8"/>
       <c r="K89" s="116" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="L89" s="4"/>
       <c r="M89" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N89" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O89" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P89" s="14"/>
     </row>
     <row r="90" spans="1:16">
       <c r="A90" s="10" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="B90" s="18" t="s">
         <v>89</v>
@@ -12905,10 +12908,10 @@
         <v>120</v>
       </c>
       <c r="G90" s="18" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H90" s="18" t="s">
         <v>1112</v>
-      </c>
-      <c r="H90" s="18" t="s">
-        <v>1113</v>
       </c>
       <c r="I90" s="18" t="s">
         <v>49</v>
@@ -12917,19 +12920,19 @@
       <c r="K90" s="33"/>
       <c r="L90" s="4"/>
       <c r="M90" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N90" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O90" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P90" s="14"/>
     </row>
     <row r="91" spans="1:16">
       <c r="A91" s="30" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="B91" s="18" t="s">
         <v>89</v>
@@ -12943,10 +12946,10 @@
         <v>15</v>
       </c>
       <c r="G91" s="17" t="s">
+        <v>1111</v>
+      </c>
+      <c r="H91" s="26" t="s">
         <v>1112</v>
-      </c>
-      <c r="H91" s="26" t="s">
-        <v>1113</v>
       </c>
       <c r="I91" s="18" t="s">
         <v>49</v>
@@ -12955,19 +12958,19 @@
       <c r="K91" s="33"/>
       <c r="L91" s="4"/>
       <c r="M91" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N91" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O91" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P91" s="14"/>
     </row>
     <row r="92" spans="1:16">
       <c r="A92" s="30" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="B92" s="36" t="s">
         <v>89</v>
@@ -12985,23 +12988,23 @@
       </c>
       <c r="J92" s="114"/>
       <c r="K92" s="114" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="L92" s="4"/>
       <c r="M92" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N92" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O92" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P92" s="14"/>
     </row>
     <row r="93" spans="1:16" ht="36">
       <c r="A93" s="30" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B93" s="26" t="s">
         <v>66</v>
@@ -13023,17 +13026,17 @@
       </c>
       <c r="J93" s="19"/>
       <c r="K93" s="33" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="L93" s="4"/>
       <c r="M93" s="5" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="N93" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O93" s="14" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="P93" s="14"/>
     </row>
@@ -13579,7 +13582,7 @@
     </row>
     <row r="14" spans="1:16" ht="24">
       <c r="A14" s="10" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B14" s="26" t="s">
         <v>584</v>
@@ -13590,7 +13593,7 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="26" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>15</v>
@@ -13617,7 +13620,7 @@
     </row>
     <row r="15" spans="1:16">
       <c r="A15" s="48" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="B15" s="26"/>
       <c r="C15" s="8"/>
@@ -20789,7 +20792,7 @@
       <c r="I2" s="25"/>
       <c r="J2" s="49"/>
       <c r="K2" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L2" s="5"/>
       <c r="M2" s="14" t="s">
@@ -20827,7 +20830,7 @@
       </c>
       <c r="J3" s="49"/>
       <c r="K3" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>57</v>
@@ -20865,7 +20868,7 @@
       <c r="I4" s="8"/>
       <c r="J4" s="49"/>
       <c r="K4" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L4" s="5" t="s">
         <v>71</v>
@@ -20903,7 +20906,7 @@
       <c r="I5" s="8"/>
       <c r="J5" s="49"/>
       <c r="K5" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>57</v>
@@ -20943,7 +20946,7 @@
       </c>
       <c r="J6" s="49"/>
       <c r="K6" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="14" t="s">
@@ -20977,7 +20980,7 @@
       <c r="I7" s="17"/>
       <c r="J7" s="49"/>
       <c r="K7" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>57</v>
@@ -21013,7 +21016,7 @@
       <c r="I8" s="17"/>
       <c r="J8" s="49"/>
       <c r="K8" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>71</v>
@@ -21053,7 +21056,7 @@
       </c>
       <c r="J9" s="49"/>
       <c r="K9" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>71</v>
@@ -21089,7 +21092,7 @@
       <c r="I10" s="8"/>
       <c r="J10" s="49"/>
       <c r="K10" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>71</v>
@@ -21127,7 +21130,7 @@
       </c>
       <c r="J11" s="49"/>
       <c r="K11" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>71</v>
@@ -21163,7 +21166,7 @@
       </c>
       <c r="J12" s="49"/>
       <c r="K12" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L12" s="5" t="s">
         <v>51</v>
@@ -21200,7 +21203,7 @@
       <c r="I13" s="8"/>
       <c r="J13" s="49"/>
       <c r="K13" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>57</v>
@@ -21230,7 +21233,7 @@
       <c r="I14" s="8"/>
       <c r="J14" s="49"/>
       <c r="K14" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="14" t="s">
@@ -21264,7 +21267,7 @@
       </c>
       <c r="J15" s="49"/>
       <c r="K15" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L15" s="5" t="s">
         <v>71</v>
@@ -21302,7 +21305,7 @@
       <c r="I16" s="17"/>
       <c r="J16" s="49"/>
       <c r="K16" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L16" s="5" t="s">
         <v>71</v>
@@ -21342,7 +21345,7 @@
       </c>
       <c r="J17" s="49"/>
       <c r="K17" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L17" s="5" t="s">
         <v>71</v>
@@ -21372,7 +21375,7 @@
       <c r="I18" s="8"/>
       <c r="J18" s="49"/>
       <c r="K18" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L18" s="5"/>
       <c r="M18" s="14" t="s">
@@ -21398,7 +21401,7 @@
       <c r="I19" s="8"/>
       <c r="J19" s="49"/>
       <c r="K19" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L19" s="5"/>
       <c r="M19" s="14" t="s">
@@ -21436,7 +21439,7 @@
       </c>
       <c r="J20" s="49"/>
       <c r="K20" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L20" s="5" t="s">
         <v>71</v>
@@ -21474,7 +21477,7 @@
       </c>
       <c r="J21" s="49"/>
       <c r="K21" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L21" s="5" t="s">
         <v>71</v>
@@ -21502,7 +21505,7 @@
       <c r="I22" s="8"/>
       <c r="J22" s="49"/>
       <c r="K22" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L22" s="5"/>
       <c r="M22" s="14" t="s">
@@ -21538,7 +21541,7 @@
       </c>
       <c r="J23" s="49"/>
       <c r="K23" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>71</v>
@@ -21578,7 +21581,7 @@
       </c>
       <c r="J24" s="49"/>
       <c r="K24" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L24" s="5" t="s">
         <v>71</v>
@@ -21612,7 +21615,7 @@
       <c r="I25" s="8"/>
       <c r="J25" s="49"/>
       <c r="K25" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>71</v>
@@ -21640,7 +21643,7 @@
       </c>
       <c r="J26" s="49"/>
       <c r="K26" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L26" s="5"/>
       <c r="M26" s="14" t="s">
@@ -21666,7 +21669,7 @@
       </c>
       <c r="J27" s="49"/>
       <c r="K27" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L27" s="5"/>
       <c r="M27" s="14" t="s">
@@ -21702,7 +21705,7 @@
       </c>
       <c r="J28" s="49"/>
       <c r="K28" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L28" s="5" t="s">
         <v>71</v>
@@ -21738,7 +21741,7 @@
       <c r="I29" s="8"/>
       <c r="J29" s="49"/>
       <c r="K29" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L29" s="5" t="s">
         <v>140</v>
@@ -21778,7 +21781,7 @@
       <c r="I30" s="1"/>
       <c r="J30" s="49"/>
       <c r="K30" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L30" s="5" t="s">
         <v>140</v>
@@ -21820,7 +21823,7 @@
       </c>
       <c r="J31" s="49"/>
       <c r="K31" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L31" s="5" t="s">
         <v>71</v>
@@ -21858,7 +21861,7 @@
       </c>
       <c r="J32" s="49"/>
       <c r="K32" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L32" s="5" t="s">
         <v>71</v>
@@ -21898,7 +21901,7 @@
       </c>
       <c r="J33" s="49"/>
       <c r="K33" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L33" s="5" t="s">
         <v>71</v>
@@ -21938,7 +21941,7 @@
       </c>
       <c r="J34" s="49"/>
       <c r="K34" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L34" s="5" t="s">
         <v>71</v>
@@ -21974,7 +21977,7 @@
       <c r="I35" s="8"/>
       <c r="J35" s="49"/>
       <c r="K35" s="5" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="L35" s="5" t="s">
         <v>71</v>
@@ -22056,7 +22059,7 @@
       </c>
       <c r="J37" s="49"/>
       <c r="K37" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L37" s="5" t="s">
         <v>71</v>
@@ -22090,7 +22093,7 @@
       <c r="I38" s="25"/>
       <c r="J38" s="49"/>
       <c r="K38" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L38" s="5" t="s">
         <v>71</v>
@@ -22126,7 +22129,7 @@
       </c>
       <c r="J39" s="49"/>
       <c r="K39" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L39" s="5" t="s">
         <v>71</v>
@@ -22160,7 +22163,7 @@
       <c r="I40" s="25"/>
       <c r="J40" s="49"/>
       <c r="K40" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L40" s="5" t="s">
         <v>71</v>
@@ -22194,7 +22197,7 @@
       <c r="I41" s="25"/>
       <c r="J41" s="49"/>
       <c r="K41" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L41" s="5" t="s">
         <v>71</v>
@@ -22228,7 +22231,7 @@
       <c r="I42" s="25"/>
       <c r="J42" s="49"/>
       <c r="K42" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L42" s="5" t="s">
         <v>71</v>
@@ -22262,7 +22265,7 @@
       <c r="I43" s="25"/>
       <c r="J43" s="49"/>
       <c r="K43" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L43" s="5" t="s">
         <v>71</v>
@@ -22296,7 +22299,7 @@
       <c r="I44" s="25"/>
       <c r="J44" s="49"/>
       <c r="K44" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L44" s="5" t="s">
         <v>71</v>
@@ -22332,7 +22335,7 @@
       </c>
       <c r="J45" s="49"/>
       <c r="K45" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>71</v>
@@ -22366,7 +22369,7 @@
       <c r="I46" s="25"/>
       <c r="J46" s="49"/>
       <c r="K46" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>71</v>
@@ -22400,7 +22403,7 @@
       <c r="I47" s="25"/>
       <c r="J47" s="49"/>
       <c r="K47" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L47" s="5" t="s">
         <v>71</v>
@@ -22434,7 +22437,7 @@
       <c r="I48" s="25"/>
       <c r="J48" s="49"/>
       <c r="K48" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L48" s="5" t="s">
         <v>71</v>
@@ -22470,7 +22473,7 @@
       <c r="I49" s="25"/>
       <c r="J49" s="49"/>
       <c r="K49" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L49" s="5" t="s">
         <v>71</v>
@@ -22506,7 +22509,7 @@
       <c r="I50" s="25"/>
       <c r="J50" s="49"/>
       <c r="K50" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L50" s="5" t="s">
         <v>71</v>
@@ -22540,7 +22543,7 @@
       <c r="I51" s="25"/>
       <c r="J51" s="49"/>
       <c r="K51" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>71</v>
@@ -22574,7 +22577,7 @@
       <c r="I52" s="59"/>
       <c r="J52" s="49"/>
       <c r="K52" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>71</v>
@@ -22608,7 +22611,7 @@
       <c r="I53" s="25"/>
       <c r="J53" s="49"/>
       <c r="K53" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>71</v>
@@ -22642,7 +22645,7 @@
       <c r="I54" s="59"/>
       <c r="J54" s="49"/>
       <c r="K54" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L54" s="5" t="s">
         <v>71</v>
@@ -22678,7 +22681,7 @@
       </c>
       <c r="J55" s="49"/>
       <c r="K55" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L55" s="5" t="s">
         <v>71</v>
@@ -22714,7 +22717,7 @@
       </c>
       <c r="J56" s="49"/>
       <c r="K56" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L56" s="5" t="s">
         <v>71</v>
@@ -22750,7 +22753,7 @@
       </c>
       <c r="J57" s="49"/>
       <c r="K57" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L57" s="5" t="s">
         <v>71</v>
@@ -22786,7 +22789,7 @@
       </c>
       <c r="J58" s="49"/>
       <c r="K58" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L58" s="5" t="s">
         <v>71</v>
@@ -22822,7 +22825,7 @@
       </c>
       <c r="J59" s="49"/>
       <c r="K59" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L59" s="5" t="s">
         <v>71</v>
@@ -22858,7 +22861,7 @@
       </c>
       <c r="J60" s="49"/>
       <c r="K60" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L60" s="5" t="s">
         <v>71</v>
@@ -22894,7 +22897,7 @@
       </c>
       <c r="J61" s="49"/>
       <c r="K61" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L61" s="5" t="s">
         <v>71</v>
@@ -22930,7 +22933,7 @@
       </c>
       <c r="J62" s="49"/>
       <c r="K62" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L62" s="5" t="s">
         <v>71</v>
@@ -22966,7 +22969,7 @@
       </c>
       <c r="J63" s="49"/>
       <c r="K63" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L63" s="5" t="s">
         <v>71</v>
@@ -23000,7 +23003,7 @@
       <c r="I64" s="25"/>
       <c r="J64" s="49"/>
       <c r="K64" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L64" s="5" t="s">
         <v>71</v>
@@ -23036,7 +23039,7 @@
       <c r="I65" s="25"/>
       <c r="J65" s="49"/>
       <c r="K65" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L65" s="5" t="s">
         <v>71</v>
@@ -23072,7 +23075,7 @@
       <c r="I66" s="25"/>
       <c r="J66" s="49"/>
       <c r="K66" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L66" s="5" t="s">
         <v>71</v>
@@ -23112,7 +23115,7 @@
       </c>
       <c r="J67" s="49"/>
       <c r="K67" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L67" s="5" t="s">
         <v>71</v>
@@ -23148,7 +23151,7 @@
       <c r="I68" s="25"/>
       <c r="J68" s="49"/>
       <c r="K68" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L68" s="5" t="s">
         <v>71</v>
@@ -23184,7 +23187,7 @@
       </c>
       <c r="J69" s="49"/>
       <c r="K69" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L69" s="5" t="s">
         <v>71</v>
@@ -23220,7 +23223,7 @@
       </c>
       <c r="J70" s="49"/>
       <c r="K70" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L70" s="5" t="s">
         <v>71</v>
@@ -23256,7 +23259,7 @@
       </c>
       <c r="J71" s="49"/>
       <c r="K71" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L71" s="5" t="s">
         <v>71</v>
@@ -23292,7 +23295,7 @@
       </c>
       <c r="J72" s="49"/>
       <c r="K72" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L72" s="5" t="s">
         <v>71</v>
@@ -23328,7 +23331,7 @@
       </c>
       <c r="J73" s="49"/>
       <c r="K73" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L73" s="5" t="s">
         <v>71</v>
@@ -23364,7 +23367,7 @@
       </c>
       <c r="J74" s="49"/>
       <c r="K74" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L74" s="5" t="s">
         <v>71</v>
@@ -23400,7 +23403,7 @@
       </c>
       <c r="J75" s="49"/>
       <c r="K75" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L75" s="5" t="s">
         <v>71</v>
@@ -23436,7 +23439,7 @@
       </c>
       <c r="J76" s="49"/>
       <c r="K76" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L76" s="5" t="s">
         <v>71</v>
@@ -23472,7 +23475,7 @@
       </c>
       <c r="J77" s="49"/>
       <c r="K77" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L77" s="5" t="s">
         <v>71</v>
@@ -23508,7 +23511,7 @@
       </c>
       <c r="J78" s="49"/>
       <c r="K78" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L78" s="5" t="s">
         <v>71</v>
@@ -23544,7 +23547,7 @@
       </c>
       <c r="J79" s="49"/>
       <c r="K79" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L79" s="5" t="s">
         <v>71</v>
@@ -23580,7 +23583,7 @@
       </c>
       <c r="J80" s="49"/>
       <c r="K80" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L80" s="5" t="s">
         <v>71</v>
@@ -23616,7 +23619,7 @@
       </c>
       <c r="J81" s="49"/>
       <c r="K81" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L81" s="5" t="s">
         <v>71</v>
@@ -23652,7 +23655,7 @@
       <c r="I82" s="25"/>
       <c r="J82" s="49"/>
       <c r="K82" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L82" s="5" t="s">
         <v>71</v>
@@ -23688,7 +23691,7 @@
       </c>
       <c r="J83" s="49"/>
       <c r="K83" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L83" s="5" t="s">
         <v>71</v>
@@ -23724,7 +23727,7 @@
       <c r="I84" s="25"/>
       <c r="J84" s="49"/>
       <c r="K84" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L84" s="5" t="s">
         <v>71</v>
@@ -23760,7 +23763,7 @@
       </c>
       <c r="J85" s="49"/>
       <c r="K85" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L85" s="5" t="s">
         <v>71</v>
@@ -23796,7 +23799,7 @@
       <c r="I86" s="25"/>
       <c r="J86" s="49"/>
       <c r="K86" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L86" s="5" t="s">
         <v>71</v>
@@ -23830,7 +23833,7 @@
       <c r="I87" s="59"/>
       <c r="J87" s="49"/>
       <c r="K87" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L87" s="5" t="s">
         <v>71</v>
@@ -23868,7 +23871,7 @@
       </c>
       <c r="J88" s="49"/>
       <c r="K88" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L88" s="5" t="s">
         <v>71</v>
@@ -23904,7 +23907,7 @@
       </c>
       <c r="J89" s="49"/>
       <c r="K89" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L89" s="5" t="s">
         <v>71</v>
@@ -23938,7 +23941,7 @@
       <c r="I90" s="25"/>
       <c r="J90" s="49"/>
       <c r="K90" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L90" s="5" t="s">
         <v>71</v>
@@ -23974,7 +23977,7 @@
       </c>
       <c r="J91" s="49"/>
       <c r="K91" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L91" s="5" t="s">
         <v>71</v>
@@ -24008,7 +24011,7 @@
       <c r="I92" s="25"/>
       <c r="J92" s="49"/>
       <c r="K92" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L92" s="5" t="s">
         <v>71</v>
@@ -24044,7 +24047,7 @@
       </c>
       <c r="J93" s="49"/>
       <c r="K93" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L93" s="5" t="s">
         <v>71</v>
@@ -24078,7 +24081,7 @@
       <c r="I94" s="25"/>
       <c r="J94" s="49"/>
       <c r="K94" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L94" s="5" t="s">
         <v>71</v>
@@ -24114,7 +24117,7 @@
       <c r="I95" s="25"/>
       <c r="J95" s="49"/>
       <c r="K95" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L95" s="5" t="s">
         <v>71</v>
@@ -24150,7 +24153,7 @@
       <c r="I96" s="25"/>
       <c r="J96" s="49"/>
       <c r="K96" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L96" s="5" t="s">
         <v>71</v>
@@ -24186,7 +24189,7 @@
       </c>
       <c r="J97" s="49"/>
       <c r="K97" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L97" s="5" t="s">
         <v>71</v>
@@ -24220,7 +24223,7 @@
       <c r="I98" s="25"/>
       <c r="J98" s="49"/>
       <c r="K98" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L98" s="5" t="s">
         <v>71</v>
@@ -24258,7 +24261,7 @@
       </c>
       <c r="J99" s="49"/>
       <c r="K99" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L99" s="5" t="s">
         <v>71</v>
@@ -24296,7 +24299,7 @@
       </c>
       <c r="J100" s="49"/>
       <c r="K100" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L100" s="5" t="s">
         <v>71</v>
@@ -24330,7 +24333,7 @@
       <c r="I101" s="25"/>
       <c r="J101" s="49"/>
       <c r="K101" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L101" s="5" t="s">
         <v>71</v>
@@ -24368,7 +24371,7 @@
       </c>
       <c r="J102" s="49"/>
       <c r="K102" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L102" s="5" t="s">
         <v>71</v>
@@ -24404,7 +24407,7 @@
       <c r="I103" s="59"/>
       <c r="J103" s="49"/>
       <c r="K103" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L103" s="5" t="s">
         <v>71</v>
@@ -24440,7 +24443,7 @@
       </c>
       <c r="J104" s="49"/>
       <c r="K104" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L104" s="5" t="s">
         <v>71</v>
@@ -24476,7 +24479,7 @@
       </c>
       <c r="J105" s="49"/>
       <c r="K105" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L105" s="5" t="s">
         <v>71</v>
@@ -24512,7 +24515,7 @@
       </c>
       <c r="J106" s="49"/>
       <c r="K106" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L106" s="5" t="s">
         <v>71</v>
@@ -24548,7 +24551,7 @@
       </c>
       <c r="J107" s="49"/>
       <c r="K107" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L107" s="5" t="s">
         <v>71</v>
@@ -24584,7 +24587,7 @@
       </c>
       <c r="J108" s="49"/>
       <c r="K108" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L108" s="5" t="s">
         <v>71</v>
@@ -24620,7 +24623,7 @@
       </c>
       <c r="J109" s="49"/>
       <c r="K109" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L109" s="5" t="s">
         <v>71</v>
@@ -24656,7 +24659,7 @@
       </c>
       <c r="J110" s="49"/>
       <c r="K110" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L110" s="5" t="s">
         <v>71</v>
@@ -24692,7 +24695,7 @@
       </c>
       <c r="J111" s="49"/>
       <c r="K111" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L111" s="5" t="s">
         <v>71</v>
@@ -24728,7 +24731,7 @@
       </c>
       <c r="J112" s="49"/>
       <c r="K112" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L112" s="5" t="s">
         <v>71</v>
@@ -24764,7 +24767,7 @@
       </c>
       <c r="J113" s="49"/>
       <c r="K113" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L113" s="5" t="s">
         <v>71</v>
@@ -24798,7 +24801,7 @@
       <c r="I114" s="25"/>
       <c r="J114" s="49"/>
       <c r="K114" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L114" s="5" t="s">
         <v>71</v>
@@ -24834,7 +24837,7 @@
       </c>
       <c r="J115" s="49"/>
       <c r="K115" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L115" s="5" t="s">
         <v>71</v>
@@ -24868,7 +24871,7 @@
       <c r="I116" s="25"/>
       <c r="J116" s="49"/>
       <c r="K116" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L116" s="5" t="s">
         <v>71</v>
@@ -24902,7 +24905,7 @@
       <c r="I117" s="25"/>
       <c r="J117" s="49"/>
       <c r="K117" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L117" s="5" t="s">
         <v>71</v>
@@ -24938,7 +24941,7 @@
       </c>
       <c r="J118" s="49"/>
       <c r="K118" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L118" s="5" t="s">
         <v>71</v>
@@ -24974,7 +24977,7 @@
       </c>
       <c r="J119" s="49"/>
       <c r="K119" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L119" s="5" t="s">
         <v>71</v>
@@ -25008,7 +25011,7 @@
       <c r="I120" s="59"/>
       <c r="J120" s="49"/>
       <c r="K120" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L120" s="5" t="s">
         <v>71</v>
@@ -25044,7 +25047,7 @@
       </c>
       <c r="J121" s="49"/>
       <c r="K121" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L121" s="5" t="s">
         <v>71</v>
@@ -25080,7 +25083,7 @@
       </c>
       <c r="J122" s="49"/>
       <c r="K122" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L122" s="5" t="s">
         <v>71</v>
@@ -25116,7 +25119,7 @@
       </c>
       <c r="J123" s="49"/>
       <c r="K123" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L123" s="5" t="s">
         <v>71</v>
@@ -25152,7 +25155,7 @@
       </c>
       <c r="J124" s="49"/>
       <c r="K124" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L124" s="5" t="s">
         <v>71</v>
@@ -25188,7 +25191,7 @@
       </c>
       <c r="J125" s="49"/>
       <c r="K125" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L125" s="5" t="s">
         <v>71</v>
@@ -25224,7 +25227,7 @@
       </c>
       <c r="J126" s="49"/>
       <c r="K126" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L126" s="5" t="s">
         <v>71</v>
@@ -25260,7 +25263,7 @@
       </c>
       <c r="J127" s="49"/>
       <c r="K127" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L127" s="5" t="s">
         <v>71</v>
@@ -25296,7 +25299,7 @@
       </c>
       <c r="J128" s="49"/>
       <c r="K128" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L128" s="5" t="s">
         <v>71</v>
@@ -25332,7 +25335,7 @@
       </c>
       <c r="J129" s="49"/>
       <c r="K129" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L129" s="5" t="s">
         <v>71</v>
@@ -25368,7 +25371,7 @@
       </c>
       <c r="J130" s="49"/>
       <c r="K130" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L130" s="5" t="s">
         <v>71</v>
@@ -25404,7 +25407,7 @@
       <c r="I131" s="25"/>
       <c r="J131" s="49"/>
       <c r="K131" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L131" s="5" t="s">
         <v>71</v>
@@ -25440,7 +25443,7 @@
       </c>
       <c r="J132" s="49"/>
       <c r="K132" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L132" s="5" t="s">
         <v>71</v>
@@ -25476,7 +25479,7 @@
       <c r="I133" s="25"/>
       <c r="J133" s="49"/>
       <c r="K133" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L133" s="5" t="s">
         <v>71</v>
@@ -25512,7 +25515,7 @@
       </c>
       <c r="J134" s="49"/>
       <c r="K134" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L134" s="5" t="s">
         <v>71</v>
@@ -25548,7 +25551,7 @@
       <c r="I135" s="25"/>
       <c r="J135" s="49"/>
       <c r="K135" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L135" s="5" t="s">
         <v>71</v>
@@ -25582,7 +25585,7 @@
       <c r="I136" s="59"/>
       <c r="J136" s="49"/>
       <c r="K136" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L136" s="5" t="s">
         <v>71</v>
@@ -25616,7 +25619,7 @@
       <c r="I137" s="25"/>
       <c r="J137" s="49"/>
       <c r="K137" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L137" s="5" t="s">
         <v>71</v>
@@ -25650,7 +25653,7 @@
       <c r="I138" s="25"/>
       <c r="J138" s="49"/>
       <c r="K138" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L138" s="5" t="s">
         <v>71</v>
@@ -25684,7 +25687,7 @@
       <c r="I139" s="25"/>
       <c r="J139" s="49"/>
       <c r="K139" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L139" s="5" t="s">
         <v>71</v>
@@ -25718,7 +25721,7 @@
       <c r="I140" s="25"/>
       <c r="J140" s="49"/>
       <c r="K140" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L140" s="5" t="s">
         <v>71</v>
@@ -25754,7 +25757,7 @@
       </c>
       <c r="J141" s="49"/>
       <c r="K141" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L141" s="5" t="s">
         <v>71</v>
@@ -25788,7 +25791,7 @@
       <c r="I142" s="25"/>
       <c r="J142" s="49"/>
       <c r="K142" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L142" s="5" t="s">
         <v>71</v>
@@ -25822,7 +25825,7 @@
       <c r="I143" s="25"/>
       <c r="J143" s="49"/>
       <c r="K143" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L143" s="5" t="s">
         <v>71</v>
@@ -25858,7 +25861,7 @@
       </c>
       <c r="J144" s="49"/>
       <c r="K144" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L144" s="5" t="s">
         <v>71</v>
@@ -25894,7 +25897,7 @@
       </c>
       <c r="J145" s="49"/>
       <c r="K145" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L145" s="5" t="s">
         <v>71</v>
@@ -25930,7 +25933,7 @@
       </c>
       <c r="J146" s="49"/>
       <c r="K146" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L146" s="5" t="s">
         <v>71</v>
@@ -25966,7 +25969,7 @@
       </c>
       <c r="J147" s="49"/>
       <c r="K147" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L147" s="5" t="s">
         <v>71</v>
@@ -26002,7 +26005,7 @@
       </c>
       <c r="J148" s="49"/>
       <c r="K148" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L148" s="5" t="s">
         <v>71</v>
@@ -26038,7 +26041,7 @@
       </c>
       <c r="J149" s="49"/>
       <c r="K149" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L149" s="5" t="s">
         <v>71</v>
@@ -26074,7 +26077,7 @@
       </c>
       <c r="J150" s="49"/>
       <c r="K150" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L150" s="5" t="s">
         <v>71</v>
@@ -26110,7 +26113,7 @@
       </c>
       <c r="J151" s="49"/>
       <c r="K151" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L151" s="5" t="s">
         <v>71</v>
@@ -26146,7 +26149,7 @@
       </c>
       <c r="J152" s="49"/>
       <c r="K152" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L152" s="5" t="s">
         <v>71</v>
@@ -26182,7 +26185,7 @@
       </c>
       <c r="J153" s="49"/>
       <c r="K153" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L153" s="5" t="s">
         <v>71</v>
@@ -26216,7 +26219,7 @@
       <c r="I154" s="59"/>
       <c r="J154" s="56"/>
       <c r="K154" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L154" s="5" t="s">
         <v>71</v>
@@ -26250,7 +26253,7 @@
       <c r="I155" s="33"/>
       <c r="J155" s="56"/>
       <c r="K155" s="5" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="L155" s="5" t="s">
         <v>71</v>
@@ -26734,7 +26737,7 @@
     </row>
     <row r="10" spans="1:16" ht="24">
       <c r="A10" s="67" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>779</v>
@@ -26748,14 +26751,14 @@
         <v>347</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="H10" s="13"/>
       <c r="I10" s="5" t="s">
         <v>49</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="K10" s="13"/>
       <c r="L10" s="59"/>
@@ -27830,7 +27833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="24">
+    <row r="17" spans="1:16">
       <c r="A17" s="85" t="s">
         <v>602</v>
       </c>
@@ -28644,7 +28647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="24">
+    <row r="38" spans="1:16">
       <c r="A38" s="85" t="s">
         <v>638</v>
       </c>
@@ -29451,7 +29454,7 @@
         <v>49</v>
       </c>
       <c r="J58" s="8" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="K58" s="4"/>
       <c r="L58" s="4"/>
@@ -29492,7 +29495,7 @@
         <v>49</v>
       </c>
       <c r="J59" s="8" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="K59" s="4"/>
       <c r="L59" s="4"/>
@@ -29533,7 +29536,7 @@
         <v>49</v>
       </c>
       <c r="J60" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K60" s="4"/>
       <c r="L60" s="4"/>
@@ -29574,7 +29577,7 @@
         <v>49</v>
       </c>
       <c r="J61" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K61" s="4"/>
       <c r="L61" s="4"/>
@@ -29615,7 +29618,7 @@
         <v>49</v>
       </c>
       <c r="J62" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K62" s="4"/>
       <c r="L62" s="4"/>
@@ -29656,7 +29659,7 @@
         <v>49</v>
       </c>
       <c r="J63" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K63" s="4"/>
       <c r="L63" s="4"/>
@@ -29697,7 +29700,7 @@
         <v>49</v>
       </c>
       <c r="J64" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K64" s="4"/>
       <c r="L64" s="4"/>
@@ -29738,7 +29741,7 @@
         <v>49</v>
       </c>
       <c r="J65" s="8" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="K65" s="4"/>
       <c r="L65" s="4"/>
@@ -29862,7 +29865,7 @@
         <v>49</v>
       </c>
       <c r="J68" s="8" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="K68" s="4"/>
       <c r="L68" s="4"/>
@@ -29903,7 +29906,7 @@
         <v>49</v>
       </c>
       <c r="J69" s="8" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="K69" s="4"/>
       <c r="L69" s="4"/>
@@ -29944,7 +29947,7 @@
         <v>49</v>
       </c>
       <c r="J70" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K70" s="4"/>
       <c r="L70" s="4"/>
@@ -29985,7 +29988,7 @@
         <v>49</v>
       </c>
       <c r="J71" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K71" s="4"/>
       <c r="L71" s="4"/>
@@ -30026,7 +30029,7 @@
         <v>49</v>
       </c>
       <c r="J72" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K72" s="4"/>
       <c r="L72" s="4"/>
@@ -30067,7 +30070,7 @@
         <v>49</v>
       </c>
       <c r="J73" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K73" s="4"/>
       <c r="L73" s="4"/>
@@ -30108,7 +30111,7 @@
         <v>49</v>
       </c>
       <c r="J74" s="8" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="K74" s="4"/>
       <c r="L74" s="4"/>
@@ -30149,7 +30152,7 @@
         <v>49</v>
       </c>
       <c r="J75" s="8" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="K75" s="4"/>
       <c r="L75" s="4"/>

</xml_diff>

<commit_message>
Added oxygen transport and utilization metrics to blood chemistry data.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/SystemValidationData.xlsx
+++ b/data/human/adult/validation/SystemValidationData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{271B74B7-C4C6-4E33-8098-20A5AB5D62BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C04C3775-BD01-4677-B3C4-B97284B998D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="30" windowWidth="28770" windowHeight="17250" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20475" yWindow="3300" windowWidth="34530" windowHeight="26775" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6617" uniqueCount="1195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6670" uniqueCount="1209">
   <si>
     <t>Patient Inputs</t>
   </si>
@@ -3757,6 +3757,48 @@
   </si>
   <si>
     <t>Thresholds</t>
+  </si>
+  <si>
+    <t>ArterialOxygenContent</t>
+  </si>
+  <si>
+    <t>ArteriovenousOxygenDifference</t>
+  </si>
+  <si>
+    <t>MixedVenousOxygenContent</t>
+  </si>
+  <si>
+    <t>OxygenDelivery</t>
+  </si>
+  <si>
+    <t>OxygenDeliveryToOxygenConsumptionRatio</t>
+  </si>
+  <si>
+    <t>Between 4:1 and 5:1</t>
+  </si>
+  <si>
+    <t>[900,1100]</t>
+  </si>
+  <si>
+    <t>ApparentOxygenConsumption</t>
+  </si>
+  <si>
+    <t>18-20 mL O2/dL blood = 18-20%</t>
+  </si>
+  <si>
+    <t>4-5 mL O2/dL blood = 4-5%</t>
+  </si>
+  <si>
+    <t>13-15 mL O2/dL blood = 13-15%</t>
+  </si>
+  <si>
+    <t>[0.18,0.20]</t>
+  </si>
+  <si>
+    <t>[0.04-0.05]</t>
+  </si>
+  <si>
+    <t>[0.13,0.15]</t>
   </si>
 </sst>
 </file>
@@ -13265,7 +13307,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AMH81"/>
+  <dimension ref="A1:AMH87"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.140625" style="1" customWidth="1"/>
@@ -13341,21 +13383,21 @@
     </row>
     <row r="2" spans="1:17">
       <c r="A2" s="10" t="s">
-        <v>44</v>
+        <v>1202</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
-      <c r="F2" s="8" t="s">
-        <v>47</v>
+      <c r="F2" s="8">
+        <v>250</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="H2" s="8"/>
       <c r="I2" s="8" t="s">
@@ -13380,46 +13422,46 @@
     </row>
     <row r="3" spans="1:17">
       <c r="A3" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>54</v>
-      </c>
+        <v>1195</v>
+      </c>
+      <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
-      <c r="F3" s="8">
-        <v>1050</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>56</v>
-      </c>
+      <c r="F3" s="2" t="s">
+        <v>1206</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="8"/>
       <c r="I3" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J3" s="8"/>
+      <c r="J3" s="8" t="s">
+        <v>1203</v>
+      </c>
       <c r="K3" s="12"/>
       <c r="L3" s="13"/>
       <c r="M3" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="O3" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P3" s="14"/>
+      <c r="P3" s="14">
+        <v>2</v>
+      </c>
       <c r="Q3" s="14"/>
     </row>
-    <row r="4" spans="1:17" ht="24">
+    <row r="4" spans="1:17">
       <c r="A4" s="10" t="s">
-        <v>58</v>
+        <v>1196</v>
       </c>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
@@ -13428,20 +13470,20 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>61</v>
-      </c>
+        <v>1207</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="8"/>
       <c r="I4" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="4"/>
+      <c r="J4" s="8" t="s">
+        <v>1204</v>
+      </c>
+      <c r="K4" s="12"/>
+      <c r="L4" s="13"/>
       <c r="M4" s="5" t="s">
         <v>50</v>
       </c>
@@ -13458,21 +13500,21 @@
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="10" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
-      <c r="F5" s="8">
-        <v>3617</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>64</v>
+      <c r="F5" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>48</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="8" t="s">
@@ -13485,60 +13527,58 @@
         <v>50</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="O5" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P5" s="14"/>
+      <c r="P5" s="14">
+        <v>2</v>
+      </c>
       <c r="Q5" s="14"/>
     </row>
-    <row r="6" spans="1:17" ht="24">
+    <row r="6" spans="1:17">
       <c r="A6" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>66</v>
+        <v>53</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>54</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
-      <c r="F6" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="G6" s="18" t="s">
-        <v>68</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>69</v>
+      <c r="F6" s="8">
+        <v>1050</v>
+      </c>
+      <c r="G6" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>56</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J6" s="8"/>
-      <c r="K6" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="L6" s="4"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="13"/>
       <c r="M6" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N6" s="5" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="O6" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P6" s="14">
-        <v>1</v>
-      </c>
+      <c r="P6" s="14"/>
       <c r="Q6" s="14"/>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" ht="24">
       <c r="A7" s="10" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
@@ -13546,19 +13586,21 @@
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
-      <c r="F7" s="8">
-        <v>0.13</v>
+      <c r="F7" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="H7" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>61</v>
+      </c>
       <c r="I7" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J7" s="8"/>
-      <c r="K7" s="12"/>
-      <c r="L7" s="13"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="4"/>
       <c r="M7" s="5" t="s">
         <v>50</v>
       </c>
@@ -13575,124 +13617,124 @@
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B8" s="8"/>
+        <v>62</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="C8" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8">
-        <v>0</v>
-      </c>
-      <c r="G8" s="8"/>
+        <v>3617</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="H8" s="8"/>
       <c r="I8" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J8" s="8" t="s">
-        <v>75</v>
-      </c>
+      <c r="J8" s="8"/>
       <c r="K8" s="12"/>
       <c r="L8" s="13"/>
       <c r="M8" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="N8" s="5"/>
+      <c r="N8" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="O8" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P8" s="14">
-        <v>2</v>
-      </c>
+      <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
     </row>
     <row r="9" spans="1:17" ht="24">
       <c r="A9" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="B9" s="8"/>
+        <v>65</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>66</v>
+      </c>
       <c r="C9" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="G9" s="8" t="s">
-        <v>78</v>
+        <v>67</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>68</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J9" s="8"/>
-      <c r="K9" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="L9" s="21"/>
+      <c r="K9" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="L9" s="4"/>
       <c r="M9" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="O9" s="14" t="s">
         <v>52</v>
       </c>
       <c r="P9" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q9" s="14"/>
     </row>
-    <row r="10" spans="1:17" s="1" customFormat="1" ht="12">
+    <row r="10" spans="1:17">
       <c r="A10" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>82</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
-      <c r="F10" s="22">
-        <f>Patient!C7*Patient!C11/100</f>
-        <v>826.44819998688286</v>
+      <c r="F10" s="8">
+        <v>0.13</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="H10" s="12"/>
+        <v>73</v>
+      </c>
+      <c r="H10" s="8"/>
       <c r="I10" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="K10" s="8" t="s">
-        <v>84</v>
-      </c>
+      <c r="J10" s="8"/>
+      <c r="K10" s="12"/>
       <c r="L10" s="13"/>
       <c r="M10" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N10" s="5" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="O10" s="14" t="s">
         <v>52</v>
       </c>
       <c r="P10" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" s="14"/>
     </row>
-    <row r="11" spans="1:17" ht="24">
+    <row r="11" spans="1:17">
       <c r="A11" s="10" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
@@ -13700,27 +13742,23 @@
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
-      <c r="F11" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>87</v>
-      </c>
+      <c r="F11" s="8">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
       <c r="I11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="4"/>
+      <c r="J11" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="12"/>
+      <c r="L11" s="13"/>
       <c r="M11" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="N11" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="N11" s="5"/>
       <c r="O11" s="14" t="s">
         <v>52</v>
       </c>
@@ -13729,79 +13767,74 @@
       </c>
       <c r="Q11" s="14"/>
     </row>
-    <row r="12" spans="1:17" ht="27.75" customHeight="1">
+    <row r="12" spans="1:17" ht="24">
       <c r="A12" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>89</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="B12" s="8"/>
       <c r="C12" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
-      <c r="F12" s="20" t="s">
-        <v>90</v>
+      <c r="F12" s="8" t="s">
+        <v>77</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="H12" s="8"/>
+        <v>78</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>79</v>
+      </c>
       <c r="I12" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
+      <c r="K12" s="20" t="s">
+        <v>80</v>
+      </c>
       <c r="L12" s="21"/>
       <c r="M12" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N12" s="5" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="O12" s="14" t="s">
         <v>52</v>
       </c>
       <c r="P12" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q12" s="14"/>
     </row>
-    <row r="13" spans="1:17" ht="27.75" customHeight="1">
+    <row r="13" spans="1:17" s="1" customFormat="1" ht="12">
       <c r="A13" s="10" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
-      <c r="F13" s="23">
-        <f>Patient!C7*(1-Patient!C11/34)</f>
-        <v>3078.9246666177987</v>
+      <c r="F13" s="22">
+        <f>Patient!C7*Patient!C11/100</f>
+        <v>826.44819998688286</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>93</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="H13" s="12"/>
       <c r="I13" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J13" s="8" t="s">
-        <v>94</v>
-      </c>
       <c r="K13" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="L13" s="21" t="s">
-        <v>96</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="L13" s="13"/>
       <c r="M13" s="5" t="s">
         <v>50</v>
       </c>
@@ -13811,72 +13844,92 @@
       <c r="O13" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P13" s="14"/>
+      <c r="P13" s="14">
+        <v>1</v>
+      </c>
       <c r="Q13" s="14"/>
     </row>
-    <row r="14" spans="1:17" ht="24">
+    <row r="14" spans="1:17">
       <c r="A14" s="10" t="s">
-        <v>1169</v>
-      </c>
-      <c r="B14" s="26" t="s">
-        <v>581</v>
-      </c>
+        <v>1197</v>
+      </c>
+      <c r="B14" s="8"/>
       <c r="C14" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
-      <c r="F14" s="26" t="s">
-        <v>1170</v>
-      </c>
-      <c r="G14" s="8" t="s">
+      <c r="F14" s="8" t="s">
+        <v>1208</v>
+      </c>
+      <c r="G14" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H14" s="26"/>
+      <c r="H14" s="8"/>
       <c r="I14" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J14" s="26"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="5"/>
+      <c r="J14" s="8" t="s">
+        <v>1205</v>
+      </c>
+      <c r="K14" s="12"/>
+      <c r="L14" s="13"/>
       <c r="M14" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N14" s="5" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="O14" s="14" t="s">
         <v>52</v>
       </c>
       <c r="P14" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="14"/>
     </row>
     <row r="15" spans="1:17">
-      <c r="A15" s="48" t="s">
-        <v>1171</v>
-      </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="8"/>
+      <c r="A15" s="10" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="14"/>
-      <c r="P15" s="14"/>
+      <c r="F15" s="8" t="s">
+        <v>1201</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J15" s="8"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="O15" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="P15" s="14">
+        <v>2</v>
+      </c>
       <c r="Q15" s="14"/>
     </row>
-    <row r="16" spans="1:17" ht="24">
+    <row r="16" spans="1:17">
       <c r="A16" s="10" t="s">
-        <v>97</v>
+        <v>1199</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8" t="s">
@@ -13885,20 +13938,20 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>87</v>
-      </c>
+        <v>134</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H16" s="8"/>
       <c r="I16" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J16" s="8"/>
-      <c r="K16" s="16"/>
-      <c r="L16" s="4"/>
+      <c r="J16" s="8" t="s">
+        <v>1200</v>
+      </c>
+      <c r="K16" s="12"/>
+      <c r="L16" s="13"/>
       <c r="M16" s="5" t="s">
         <v>50</v>
       </c>
@@ -13915,110 +13968,116 @@
     </row>
     <row r="17" spans="1:17" ht="24">
       <c r="A17" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>99</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="B17" s="8"/>
       <c r="C17" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="22">
-        <f>(F10/0.000000000029)/(Patient!C7*1000)</f>
-        <v>5172413.793103449</v>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J17" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="K17" s="25"/>
-      <c r="L17" s="21"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="4"/>
       <c r="M17" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="O17" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P17" s="14"/>
+      <c r="P17" s="14">
+        <v>2</v>
+      </c>
       <c r="Q17" s="14"/>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:17" ht="27.75" customHeight="1">
       <c r="A18" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="B18" s="12"/>
+        <v>88</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="C18" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D18" s="8"/>
       <c r="E18" s="8"/>
-      <c r="F18" s="8" t="s">
-        <v>103</v>
+      <c r="F18" s="20" t="s">
+        <v>90</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>105</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="H18" s="8"/>
       <c r="I18" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J18" s="8"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="13"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="21"/>
       <c r="M18" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N18" s="5" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="O18" s="14" t="s">
         <v>52</v>
       </c>
       <c r="P18" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q18" s="14"/>
     </row>
-    <row r="19" spans="1:17">
+    <row r="19" spans="1:17" ht="27.75" customHeight="1">
       <c r="A19" s="10" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>89</v>
+        <v>17</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D19" s="8"/>
       <c r="E19" s="8"/>
-      <c r="F19" s="20" t="s">
-        <v>107</v>
+      <c r="F19" s="23">
+        <f>Patient!C7*(1-Patient!C11/34)</f>
+        <v>3078.9246666177987</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="H19" s="8"/>
+        <v>15</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>93</v>
+      </c>
       <c r="I19" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J19" s="8"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="13"/>
+      <c r="J19" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="L19" s="21" t="s">
+        <v>96</v>
+      </c>
       <c r="M19" s="5" t="s">
         <v>50</v>
       </c>
@@ -14028,158 +14087,143 @@
       <c r="O19" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P19" s="14">
-        <v>1</v>
-      </c>
+      <c r="P19" s="14"/>
       <c r="Q19" s="14"/>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" ht="24">
       <c r="A20" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>110</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
+        <v>1169</v>
+      </c>
+      <c r="B20" s="26" t="s">
+        <v>581</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
       <c r="F20" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="G20" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="H20" s="26" t="s">
-        <v>113</v>
-      </c>
+        <v>1170</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="26"/>
       <c r="I20" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J20" s="26"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="5"/>
       <c r="M20" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="O20" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="P20" s="14"/>
+      <c r="P20" s="14">
+        <v>1</v>
+      </c>
       <c r="Q20" s="14"/>
     </row>
     <row r="21" spans="1:17">
-      <c r="A21" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="8" t="s">
-        <v>46</v>
-      </c>
+      <c r="A21" s="48" t="s">
+        <v>1171</v>
+      </c>
+      <c r="B21" s="26"/>
+      <c r="C21" s="8"/>
       <c r="D21" s="8"/>
       <c r="E21" s="8"/>
-      <c r="F21" s="8">
-        <v>2.3E-3</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="H21" s="12"/>
-      <c r="I21" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J21" s="12"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="26"/>
       <c r="K21" s="8"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="N21" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="O21" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="P21" s="14">
-        <v>5</v>
-      </c>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="14"/>
+      <c r="P21" s="14"/>
       <c r="Q21" s="14"/>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" ht="24">
       <c r="A22" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="B22" s="12"/>
+        <v>97</v>
+      </c>
+      <c r="B22" s="8"/>
       <c r="C22" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D22" s="8"/>
       <c r="E22" s="8"/>
-      <c r="F22" s="8">
-        <v>1.2999999999999999E-3</v>
+      <c r="F22" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="H22" s="12"/>
+        <v>78</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>87</v>
+      </c>
       <c r="I22" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J22" s="12"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="13"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="4"/>
       <c r="M22" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N22" s="5" t="s">
-        <v>116</v>
+        <v>51</v>
       </c>
       <c r="O22" s="14" t="s">
         <v>52</v>
       </c>
       <c r="P22" s="14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Q22" s="14"/>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" ht="24">
       <c r="A23" s="10" t="s">
-        <v>118</v>
-      </c>
-      <c r="B23" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>99</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="27">
-        <v>7000</v>
-      </c>
-      <c r="G23" s="17" t="s">
-        <v>119</v>
-      </c>
-      <c r="H23" s="17" t="s">
-        <v>120</v>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="22">
+        <f>(F13/0.000000000029)/(Patient!C7*1000)</f>
+        <v>5172413.793103449</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>100</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J23" s="17"/>
-      <c r="K23" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="L23" s="4"/>
+      <c r="J23" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="K23" s="25"/>
+      <c r="L23" s="21"/>
       <c r="M23" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N23" s="5" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="O23" s="14" t="s">
         <v>52</v>
@@ -14187,86 +14231,70 @@
       <c r="P23" s="14"/>
       <c r="Q23" s="14"/>
     </row>
-    <row r="24" spans="1:17" ht="24">
-      <c r="A24" s="28" t="s">
-        <v>123</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="G24" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="H24" s="29" t="s">
-        <v>126</v>
-      </c>
-      <c r="I24" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="J24" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="L24" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="M24" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="N24" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="O24" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="P24" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q24" s="9" t="s">
-        <v>1194</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" ht="56.25">
-      <c r="A25" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>128</v>
+    <row r="24" spans="1:17">
+      <c r="A24" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B24" s="12"/>
+      <c r="C24" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J24" s="8"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="N24" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="O24" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="P24" s="14">
+        <v>3</v>
+      </c>
+      <c r="Q24" s="14"/>
+    </row>
+    <row r="25" spans="1:17">
+      <c r="A25" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>89</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D25" s="8"/>
       <c r="E25" s="8"/>
-      <c r="F25" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="G25" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="J25" s="18"/>
-      <c r="K25" s="31" t="s">
-        <v>131</v>
-      </c>
-      <c r="L25" s="4"/>
+      <c r="F25" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J25" s="8"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="13"/>
       <c r="M25" s="5" t="s">
         <v>50</v>
       </c>
@@ -14274,41 +14302,39 @@
         <v>71</v>
       </c>
       <c r="O25" s="14" t="s">
-        <v>132</v>
+        <v>52</v>
       </c>
       <c r="P25" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q25" s="14"/>
     </row>
-    <row r="26" spans="1:17" ht="22.5">
-      <c r="A26" s="30" t="s">
-        <v>133</v>
-      </c>
-      <c r="B26" s="18" t="s">
+    <row r="26" spans="1:17">
+      <c r="A26" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="C26" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="G26" s="18" t="s">
+      <c r="C26" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="G26" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="H26" s="18" t="s">
+      <c r="H26" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="I26" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="J26" s="18"/>
-      <c r="K26" s="32" t="s">
-        <v>135</v>
-      </c>
+      <c r="I26" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J26" s="26"/>
+      <c r="K26" s="4"/>
       <c r="L26" s="4"/>
       <c r="M26" s="5" t="s">
         <v>50</v>
@@ -14317,248 +14343,248 @@
         <v>71</v>
       </c>
       <c r="O26" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="P26" s="14">
-        <v>1</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="P26" s="14"/>
       <c r="Q26" s="14"/>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>110</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="B27" s="12"/>
       <c r="C27" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
-      <c r="F27" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="G27" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="H27" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="I27" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="L27" s="4"/>
+      <c r="F27" s="8">
+        <v>2.3E-3</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="H27" s="12"/>
+      <c r="I27" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J27" s="12"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="13"/>
       <c r="M27" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N27" s="5" t="s">
-        <v>140</v>
+        <v>116</v>
       </c>
       <c r="O27" s="14" t="s">
-        <v>132</v>
+        <v>52</v>
       </c>
       <c r="P27" s="14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q27" s="14"/>
     </row>
     <row r="28" spans="1:17">
       <c r="A28" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="B28" s="18" t="s">
-        <v>128</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="B28" s="12"/>
       <c r="C28" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
-      <c r="F28" s="17" t="s">
-        <v>142</v>
-      </c>
-      <c r="G28" s="18" t="s">
-        <v>143</v>
-      </c>
-      <c r="H28" s="17" t="s">
-        <v>138</v>
-      </c>
-      <c r="I28" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="J28" s="17"/>
-      <c r="K28" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="L28" s="4"/>
+      <c r="F28" s="8">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="H28" s="12"/>
+      <c r="I28" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J28" s="12"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="13"/>
       <c r="M28" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N28" s="5" t="s">
-        <v>71</v>
+        <v>116</v>
       </c>
       <c r="O28" s="14" t="s">
-        <v>132</v>
+        <v>52</v>
       </c>
       <c r="P28" s="14">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Q28" s="14"/>
     </row>
-    <row r="29" spans="1:17" ht="36">
+    <row r="29" spans="1:17">
       <c r="A29" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>146</v>
+        <v>118</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>99</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D29" s="8"/>
       <c r="E29" s="8"/>
-      <c r="F29" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="G29" s="18" t="s">
-        <v>148</v>
+      <c r="F29" s="27">
+        <v>7000</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>119</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="I29" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="I29" s="8" t="s">
         <v>49</v>
       </c>
       <c r="J29" s="17"/>
-      <c r="K29" s="8" t="s">
-        <v>150</v>
+      <c r="K29" s="16" t="s">
+        <v>121</v>
       </c>
       <c r="L29" s="4"/>
       <c r="M29" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N29" s="5" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="O29" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="P29" s="14">
-        <v>4</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="P29" s="14"/>
       <c r="Q29" s="14"/>
     </row>
     <row r="30" spans="1:17" ht="24">
-      <c r="A30" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="B30" s="17" t="s">
+      <c r="A30" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G30" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="H30" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="I30" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L30" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="M30" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N30" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="O30" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P30" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q30" s="9" t="s">
+        <v>1194</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="56.25">
+      <c r="A31" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="B31" s="18" t="s">
         <v>128</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="G30" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="H30" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="I30" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="J30" s="17"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
-      <c r="M30" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="N30" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="O30" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="P30" s="14">
-        <v>1</v>
-      </c>
-      <c r="Q30" s="14"/>
-    </row>
-    <row r="31" spans="1:17" ht="60">
-      <c r="A31" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="B31" s="17" t="s">
-        <v>155</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D31" s="8"/>
       <c r="E31" s="8"/>
-      <c r="F31" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="G31" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="H31" s="17"/>
+      <c r="F31" s="18" t="s">
+        <v>129</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="H31" s="18"/>
       <c r="I31" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J31" s="17"/>
-      <c r="K31" s="4"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="31" t="s">
+        <v>131</v>
+      </c>
       <c r="L31" s="4"/>
       <c r="M31" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N31" s="5" t="s">
-        <v>140</v>
+        <v>71</v>
       </c>
       <c r="O31" s="14" t="s">
         <v>132</v>
       </c>
       <c r="P31" s="14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q31" s="14"/>
     </row>
-    <row r="32" spans="1:17">
-      <c r="A32" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="B32" s="17" t="s">
+    <row r="32" spans="1:17" ht="22.5">
+      <c r="A32" s="30" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="C32" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="26" t="s">
-        <v>159</v>
-      </c>
-      <c r="G32" s="26" t="s">
+      <c r="C32" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="G32" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="H32" s="26" t="s">
+      <c r="H32" s="18" t="s">
         <v>113</v>
       </c>
       <c r="I32" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J32" s="17"/>
-      <c r="K32" s="4"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="32" t="s">
+        <v>135</v>
+      </c>
       <c r="L32" s="4"/>
       <c r="M32" s="5" t="s">
         <v>50</v>
@@ -14576,81 +14602,76 @@
     </row>
     <row r="33" spans="1:17">
       <c r="A33" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="B33" s="17" t="s">
-        <v>66</v>
+        <v>136</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D33" s="8"/>
       <c r="E33" s="8"/>
-      <c r="F33" s="17" t="s">
-        <v>161</v>
+      <c r="F33" s="8" t="s">
+        <v>137</v>
       </c>
       <c r="G33" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="H33" s="17"/>
+        <v>112</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>138</v>
+      </c>
       <c r="I33" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J33" s="17"/>
-      <c r="K33" s="4" t="s">
-        <v>163</v>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8" t="s">
+        <v>139</v>
       </c>
       <c r="L33" s="4"/>
       <c r="M33" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N33" s="5" t="s">
-        <v>71</v>
+        <v>140</v>
       </c>
       <c r="O33" s="14" t="s">
         <v>132</v>
       </c>
       <c r="P33" s="14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q33" s="14"/>
     </row>
-    <row r="34" spans="1:17" ht="36.75">
+    <row r="34" spans="1:17">
       <c r="A34" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>110</v>
+        <v>141</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>128</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="F34" s="14" t="str">
-        <f>IF(Patient!C7&lt;&gt;"Male",D34,E34)</f>
-        <v>[13.8,17.2]</v>
-      </c>
-      <c r="G34" s="17" t="s">
-        <v>15</v>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>143</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>167</v>
+        <v>138</v>
       </c>
       <c r="I34" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J34" s="17"/>
-      <c r="K34" s="33" t="s">
-        <v>168</v>
-      </c>
-      <c r="L34" s="21" t="s">
-        <v>169</v>
-      </c>
+      <c r="K34" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="L34" s="4"/>
       <c r="M34" s="5" t="s">
         <v>50</v>
       </c>
@@ -14665,31 +14686,33 @@
       </c>
       <c r="Q34" s="14"/>
     </row>
-    <row r="35" spans="1:17">
+    <row r="35" spans="1:17" ht="36">
       <c r="A35" s="10" t="s">
-        <v>170</v>
+        <v>145</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D35" s="8"/>
       <c r="E35" s="8"/>
-      <c r="F35" s="26">
-        <v>0.40600000000000003</v>
-      </c>
-      <c r="G35" s="17" t="s">
-        <v>162</v>
-      </c>
-      <c r="H35" s="26"/>
+      <c r="F35" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="H35" s="17" t="s">
+        <v>149</v>
+      </c>
       <c r="I35" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J35" s="26"/>
-      <c r="K35" s="4" t="s">
-        <v>171</v>
+      <c r="J35" s="17"/>
+      <c r="K35" s="8" t="s">
+        <v>150</v>
       </c>
       <c r="L35" s="4"/>
       <c r="M35" s="5" t="s">
@@ -14702,15 +14725,15 @@
         <v>132</v>
       </c>
       <c r="P35" s="14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q35" s="14"/>
     </row>
     <row r="36" spans="1:17" ht="24">
       <c r="A36" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="B36" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="B36" s="17" t="s">
         <v>128</v>
       </c>
       <c r="C36" s="8" t="s">
@@ -14718,22 +14741,20 @@
       </c>
       <c r="D36" s="8"/>
       <c r="E36" s="8"/>
-      <c r="F36" s="26" t="s">
-        <v>173</v>
+      <c r="F36" s="20" t="s">
+        <v>152</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>174</v>
-      </c>
-      <c r="H36" s="26" t="s">
-        <v>175</v>
+        <v>112</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>153</v>
       </c>
       <c r="I36" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J36" s="5"/>
-      <c r="K36" s="4" t="s">
-        <v>176</v>
-      </c>
+      <c r="J36" s="17"/>
+      <c r="K36" s="4"/>
       <c r="L36" s="4"/>
       <c r="M36" s="5" t="s">
         <v>50</v>
@@ -14745,13 +14766,13 @@
         <v>132</v>
       </c>
       <c r="P36" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q36" s="14"/>
     </row>
-    <row r="37" spans="1:17">
+    <row r="37" spans="1:17" ht="60">
       <c r="A37" s="10" t="s">
-        <v>177</v>
+        <v>154</v>
       </c>
       <c r="B37" s="17" t="s">
         <v>155</v>
@@ -14761,17 +14782,17 @@
       </c>
       <c r="D37" s="8"/>
       <c r="E37" s="8"/>
-      <c r="F37" s="26" t="s">
-        <v>178</v>
+      <c r="F37" s="8" t="s">
+        <v>156</v>
       </c>
       <c r="G37" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="H37" s="26"/>
+        <v>157</v>
+      </c>
+      <c r="H37" s="17"/>
       <c r="I37" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J37" s="5"/>
+      <c r="J37" s="17"/>
       <c r="K37" s="4"/>
       <c r="L37" s="4"/>
       <c r="M37" s="5" t="s">
@@ -14788,34 +14809,32 @@
       </c>
       <c r="Q37" s="14"/>
     </row>
-    <row r="38" spans="1:17" ht="24">
+    <row r="38" spans="1:17">
       <c r="A38" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="B38" s="18" t="s">
-        <v>128</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8" t="s">
-        <v>181</v>
-      </c>
-      <c r="G38" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="H38" s="8" t="s">
-        <v>183</v>
+        <v>158</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="G38" s="26" t="s">
+        <v>112</v>
+      </c>
+      <c r="H38" s="26" t="s">
+        <v>113</v>
       </c>
       <c r="I38" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J38" s="8"/>
-      <c r="K38" s="4" t="s">
-        <v>184</v>
-      </c>
+      <c r="J38" s="17"/>
+      <c r="K38" s="4"/>
       <c r="L38" s="4"/>
       <c r="M38" s="5" t="s">
         <v>50</v>
@@ -14827,82 +14846,87 @@
         <v>132</v>
       </c>
       <c r="P38" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q38" s="14"/>
     </row>
-    <row r="39" spans="1:17" ht="24">
+    <row r="39" spans="1:17">
       <c r="A39" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="B39" s="18" t="s">
-        <v>110</v>
+        <v>160</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>66</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D39" s="8"/>
       <c r="E39" s="8"/>
-      <c r="F39" s="8" t="s">
-        <v>186</v>
-      </c>
-      <c r="G39" s="17" t="s">
-        <v>112</v>
-      </c>
-      <c r="H39" s="8" t="s">
-        <v>187</v>
-      </c>
+      <c r="F39" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="G39" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="H39" s="17"/>
       <c r="I39" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J39" s="8"/>
-      <c r="K39" s="34" t="s">
-        <v>188</v>
+      <c r="J39" s="17"/>
+      <c r="K39" s="4" t="s">
+        <v>163</v>
       </c>
       <c r="L39" s="4"/>
       <c r="M39" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N39" s="5" t="s">
-        <v>140</v>
+        <v>71</v>
       </c>
       <c r="O39" s="14" t="s">
         <v>132</v>
       </c>
       <c r="P39" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Q39" s="14"/>
     </row>
-    <row r="40" spans="1:17">
+    <row r="40" spans="1:17" ht="36.75">
       <c r="A40" s="10" t="s">
-        <v>189</v>
-      </c>
-      <c r="B40" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="C40" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="36" t="s">
-        <v>190</v>
-      </c>
-      <c r="G40" s="36" t="s">
-        <v>112</v>
-      </c>
-      <c r="H40" s="36" t="s">
-        <v>138</v>
-      </c>
-      <c r="I40" s="36" t="s">
-        <v>49</v>
-      </c>
-      <c r="J40" s="36"/>
-      <c r="K40" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="L40" s="4"/>
+        <v>164</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="F40" s="14" t="str">
+        <f>IF(Patient!C7&lt;&gt;"Male",D40,E40)</f>
+        <v>[13.8,17.2]</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="I40" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J40" s="17"/>
+      <c r="K40" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="L40" s="21" t="s">
+        <v>169</v>
+      </c>
       <c r="M40" s="5" t="s">
         <v>50</v>
       </c>
@@ -14912,40 +14936,38 @@
       <c r="O40" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="P40" s="14"/>
+      <c r="P40" s="14">
+        <v>2</v>
+      </c>
       <c r="Q40" s="14"/>
     </row>
-    <row r="41" spans="1:17" ht="36">
+    <row r="41" spans="1:17">
       <c r="A41" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="B41" s="26" t="s">
-        <v>66</v>
+        <v>170</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>155</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D41" s="8"/>
       <c r="E41" s="8"/>
-      <c r="F41" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="G41" s="26" t="s">
-        <v>194</v>
+      <c r="F41" s="26">
+        <v>0.40600000000000003</v>
+      </c>
+      <c r="G41" s="17" t="s">
+        <v>162</v>
       </c>
       <c r="H41" s="26"/>
       <c r="I41" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="J41" s="37" t="s">
-        <v>195</v>
-      </c>
-      <c r="K41" s="38" t="s">
-        <v>196</v>
-      </c>
-      <c r="L41" s="39" t="s">
-        <v>197</v>
-      </c>
+      <c r="J41" s="26"/>
+      <c r="K41" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="L41" s="4"/>
       <c r="M41" s="5" t="s">
         <v>50</v>
       </c>
@@ -14956,128 +14978,120 @@
         <v>132</v>
       </c>
       <c r="P41" s="14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q41" s="14"/>
     </row>
     <row r="42" spans="1:17" ht="24">
-      <c r="A42" s="28" t="s">
-        <v>198</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="G42" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="H42" s="29" t="s">
-        <v>126</v>
-      </c>
-      <c r="I42" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="J42" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K42" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="L42" s="29" t="s">
-        <v>39</v>
-      </c>
-      <c r="M42" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="N42" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="O42" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="P42" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q42" s="9" t="s">
-        <v>1194</v>
-      </c>
+      <c r="A42" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="G42" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="H42" s="26" t="s">
+        <v>175</v>
+      </c>
+      <c r="I42" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J42" s="5"/>
+      <c r="K42" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="L42" s="4"/>
+      <c r="M42" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="N42" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O42" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="P42" s="14">
+        <v>3</v>
+      </c>
+      <c r="Q42" s="14"/>
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>200</v>
+        <v>177</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>155</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D43" s="8"/>
       <c r="E43" s="8"/>
-      <c r="F43" s="8">
-        <v>40</v>
-      </c>
-      <c r="G43" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H43" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="I43" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J43" s="8"/>
+      <c r="F43" s="26" t="s">
+        <v>178</v>
+      </c>
+      <c r="G43" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="H43" s="26"/>
+      <c r="I43" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J43" s="5"/>
       <c r="K43" s="4"/>
       <c r="L43" s="4"/>
       <c r="M43" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N43" s="5" t="s">
-        <v>71</v>
+        <v>140</v>
       </c>
       <c r="O43" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="P43" s="14"/>
+        <v>132</v>
+      </c>
+      <c r="P43" s="14">
+        <v>4</v>
+      </c>
       <c r="Q43" s="14"/>
     </row>
-    <row r="44" spans="1:17">
+    <row r="44" spans="1:17" ht="24">
       <c r="A44" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>200</v>
+        <v>180</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>128</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D44" s="8"/>
       <c r="E44" s="8"/>
-      <c r="F44" s="8">
-        <v>95</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>15</v>
+      <c r="F44" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="G44" s="17" t="s">
+        <v>182</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>203</v>
-      </c>
-      <c r="I44" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I44" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J44" s="8"/>
-      <c r="K44" s="4"/>
+      <c r="K44" s="4" t="s">
+        <v>184</v>
+      </c>
       <c r="L44" s="4"/>
       <c r="M44" s="5" t="s">
         <v>50</v>
@@ -15086,76 +15100,84 @@
         <v>71</v>
       </c>
       <c r="O44" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="P44" s="14"/>
+        <v>132</v>
+      </c>
+      <c r="P44" s="14">
+        <v>2</v>
+      </c>
       <c r="Q44" s="14"/>
     </row>
-    <row r="45" spans="1:17">
+    <row r="45" spans="1:17" ht="24">
       <c r="A45" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>200</v>
+        <v>185</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D45" s="8"/>
       <c r="E45" s="8"/>
-      <c r="F45" s="20">
-        <v>45</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>15</v>
+      <c r="F45" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="G45" s="17" t="s">
+        <v>112</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>201</v>
-      </c>
-      <c r="I45" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="I45" s="18" t="s">
         <v>49</v>
       </c>
       <c r="J45" s="8"/>
-      <c r="K45" s="4"/>
+      <c r="K45" s="34" t="s">
+        <v>188</v>
+      </c>
       <c r="L45" s="4"/>
       <c r="M45" s="5" t="s">
         <v>50</v>
       </c>
       <c r="N45" s="5" t="s">
-        <v>71</v>
+        <v>140</v>
       </c>
       <c r="O45" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="P45" s="14"/>
+        <v>132</v>
+      </c>
+      <c r="P45" s="14">
+        <v>3</v>
+      </c>
       <c r="Q45" s="14"/>
     </row>
     <row r="46" spans="1:17">
       <c r="A46" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
-      <c r="F46" s="20">
-        <v>40</v>
-      </c>
-      <c r="G46" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H46" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="I46" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J46" s="8"/>
-      <c r="K46" s="4"/>
+        <v>189</v>
+      </c>
+      <c r="B46" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="C46" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="36" t="s">
+        <v>190</v>
+      </c>
+      <c r="G46" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="H46" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="I46" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="J46" s="36"/>
+      <c r="K46" s="4" t="s">
+        <v>191</v>
+      </c>
       <c r="L46" s="4"/>
       <c r="M46" s="5" t="s">
         <v>50</v>
@@ -15164,38 +15186,42 @@
         <v>71</v>
       </c>
       <c r="O46" s="14" t="s">
-        <v>52</v>
+        <v>132</v>
       </c>
       <c r="P46" s="14"/>
       <c r="Q46" s="14"/>
     </row>
-    <row r="47" spans="1:17">
+    <row r="47" spans="1:17" ht="36">
       <c r="A47" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>200</v>
+        <v>192</v>
+      </c>
+      <c r="B47" s="26" t="s">
+        <v>66</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D47" s="8"/>
       <c r="E47" s="8"/>
-      <c r="F47" s="20">
-        <v>40</v>
-      </c>
-      <c r="G47" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H47" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="I47" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J47" s="8"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4"/>
+      <c r="F47" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="G47" s="26" t="s">
+        <v>194</v>
+      </c>
+      <c r="H47" s="26"/>
+      <c r="I47" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J47" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="K47" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="L47" s="39" t="s">
+        <v>197</v>
+      </c>
       <c r="M47" s="5" t="s">
         <v>50</v>
       </c>
@@ -15203,53 +15229,69 @@
         <v>71</v>
       </c>
       <c r="O47" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="P47" s="14"/>
+        <v>132</v>
+      </c>
+      <c r="P47" s="14">
+        <v>2</v>
+      </c>
       <c r="Q47" s="14"/>
     </row>
-    <row r="48" spans="1:17">
-      <c r="A48" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="20">
-        <v>104</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>206</v>
-      </c>
-      <c r="I48" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="J48" s="8"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="4"/>
-      <c r="M48" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="N48" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="O48" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="P48" s="14"/>
-      <c r="Q48" s="14"/>
+    <row r="48" spans="1:17" ht="24">
+      <c r="A48" s="28" t="s">
+        <v>198</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F48" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G48" s="29" t="s">
+        <v>125</v>
+      </c>
+      <c r="H48" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="I48" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L48" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="M48" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N48" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="O48" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P48" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q48" s="9" t="s">
+        <v>1194</v>
+      </c>
     </row>
     <row r="49" spans="1:17">
       <c r="A49" s="10" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="B49" s="8" t="s">
         <v>200</v>
@@ -15288,7 +15330,7 @@
     </row>
     <row r="50" spans="1:17">
       <c r="A50" s="10" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B50" s="8" t="s">
         <v>200</v>
@@ -15299,13 +15341,13 @@
       <c r="D50" s="8"/>
       <c r="E50" s="8"/>
       <c r="F50" s="8">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>15</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I50" s="8" t="s">
         <v>49</v>
@@ -15325,149 +15367,126 @@
       <c r="P50" s="14"/>
       <c r="Q50" s="14"/>
     </row>
-    <row r="51" spans="1:17" ht="24">
-      <c r="A51" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D51" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I51" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="J51" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="K51" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="L51" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="M51" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="N51" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="O51" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="P51" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q51" s="9" t="s">
-        <v>1194</v>
-      </c>
-    </row>
-    <row r="52" spans="1:17" ht="24">
-      <c r="A52" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B52" s="8"/>
+    <row r="51" spans="1:17">
+      <c r="A51" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="20">
+        <v>45</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H51" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="I51" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J51" s="8"/>
+      <c r="K51" s="4"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="N51" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O51" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="P51" s="14"/>
+      <c r="Q51" s="14"/>
+    </row>
+    <row r="52" spans="1:17">
+      <c r="A52" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>200</v>
+      </c>
       <c r="C52" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D52" s="8"/>
       <c r="E52" s="8"/>
-      <c r="F52" s="8" t="str">
-        <f>F4</f>
-        <v>7.2,
- [7.35,7.4]</v>
-      </c>
-      <c r="G52" s="8" t="str">
-        <f>G4</f>
-        <v>valentin2002icrp,  guyton2006medical</v>
-      </c>
-      <c r="H52" s="8" t="str">
-        <f>H4</f>
-        <v>p137                                 p384</v>
-      </c>
-      <c r="I52" s="8" t="str">
-        <f>I4</f>
-        <v>Y</v>
-      </c>
-      <c r="J52" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="K52" s="4" t="s">
-        <v>1189</v>
-      </c>
+      <c r="F52" s="20">
+        <v>40</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="I52" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J52" s="8"/>
+      <c r="K52" s="4"/>
       <c r="L52" s="4"/>
       <c r="M52" s="5" t="s">
-        <v>214</v>
+        <v>50</v>
       </c>
       <c r="N52" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O52" s="5" t="s">
-        <v>1185</v>
+      <c r="O52" s="14" t="s">
+        <v>52</v>
       </c>
       <c r="P52" s="14"/>
       <c r="Q52" s="14"/>
     </row>
     <row r="53" spans="1:17">
-      <c r="A53" s="40" t="s">
-        <v>215</v>
-      </c>
-      <c r="B53" s="18" t="s">
-        <v>45</v>
+      <c r="A53" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>200</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D53" s="8"/>
       <c r="E53" s="8"/>
-      <c r="F53" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="G53" s="18" t="s">
-        <v>112</v>
+      <c r="F53" s="20">
+        <v>40</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>15</v>
       </c>
       <c r="H53" s="8" t="s">
-        <v>138</v>
+        <v>208</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J53" s="4" t="s">
-        <v>217</v>
-      </c>
+      <c r="J53" s="8"/>
       <c r="K53" s="4"/>
       <c r="L53" s="4"/>
       <c r="M53" s="5" t="s">
-        <v>214</v>
+        <v>50</v>
       </c>
       <c r="N53" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O53" s="5" t="s">
-        <v>1185</v>
+      <c r="O53" s="14" t="s">
+        <v>52</v>
       </c>
       <c r="P53" s="14"/>
       <c r="Q53" s="14"/>
     </row>
     <row r="54" spans="1:17">
-      <c r="A54" s="40" t="s">
-        <v>218</v>
+      <c r="A54" s="10" t="s">
+        <v>209</v>
       </c>
       <c r="B54" s="8" t="s">
         <v>200</v>
@@ -15477,38 +15496,36 @@
       </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
-      <c r="F54" s="8">
-        <v>95</v>
+      <c r="F54" s="20">
+        <v>104</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>15</v>
       </c>
       <c r="H54" s="8" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J54" s="4" t="s">
-        <v>213</v>
-      </c>
+      <c r="J54" s="8"/>
       <c r="K54" s="4"/>
       <c r="L54" s="4"/>
       <c r="M54" s="5" t="s">
-        <v>214</v>
+        <v>50</v>
       </c>
       <c r="N54" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O54" s="5" t="s">
-        <v>1185</v>
+      <c r="O54" s="14" t="s">
+        <v>52</v>
       </c>
       <c r="P54" s="14"/>
       <c r="Q54" s="14"/>
     </row>
     <row r="55" spans="1:17">
-      <c r="A55" s="40" t="s">
-        <v>219</v>
+      <c r="A55" s="10" t="s">
+        <v>210</v>
       </c>
       <c r="B55" s="8" t="s">
         <v>200</v>
@@ -15530,65 +15547,63 @@
       <c r="I55" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J55" s="4" t="s">
-        <v>213</v>
-      </c>
+      <c r="J55" s="8"/>
       <c r="K55" s="4"/>
       <c r="L55" s="4"/>
       <c r="M55" s="5" t="s">
-        <v>214</v>
+        <v>50</v>
       </c>
       <c r="N55" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O55" s="5" t="s">
-        <v>1185</v>
+      <c r="O55" s="14" t="s">
+        <v>52</v>
       </c>
       <c r="P55" s="14"/>
       <c r="Q55" s="14"/>
     </row>
-    <row r="56" spans="1:17" ht="24">
-      <c r="A56" s="40" t="s">
-        <v>85</v>
-      </c>
-      <c r="B56" s="8"/>
+    <row r="56" spans="1:17">
+      <c r="A56" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>200</v>
+      </c>
       <c r="C56" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
-      <c r="F56" s="8" t="s">
-        <v>86</v>
+      <c r="F56" s="8">
+        <v>45</v>
       </c>
       <c r="G56" s="8" t="s">
-        <v>78</v>
+        <v>15</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>87</v>
+        <v>201</v>
       </c>
       <c r="I56" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J56" s="4" t="s">
-        <v>213</v>
-      </c>
+      <c r="J56" s="8"/>
       <c r="K56" s="4"/>
       <c r="L56" s="4"/>
       <c r="M56" s="5" t="s">
-        <v>214</v>
+        <v>50</v>
       </c>
       <c r="N56" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="O56" s="5" t="s">
-        <v>1185</v>
+      <c r="O56" s="14" t="s">
+        <v>52</v>
       </c>
       <c r="P56" s="14"/>
       <c r="Q56" s="14"/>
     </row>
     <row r="57" spans="1:17" ht="24">
       <c r="A57" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B57" s="9" t="s">
         <v>1</v>
@@ -15596,8 +15611,12 @@
       <c r="C57" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
+      <c r="D57" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="F57" s="9" t="s">
         <v>34</v>
       </c>
@@ -15635,262 +15654,282 @@
         <v>1194</v>
       </c>
     </row>
-    <row r="58" spans="1:17">
+    <row r="58" spans="1:17" ht="24">
       <c r="A58" s="40" t="s">
-        <v>76</v>
-      </c>
-      <c r="B58" s="4"/>
-      <c r="C58" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D58" s="5"/>
-      <c r="E58" s="5"/>
-      <c r="F58" s="14" t="str">
-        <f>F9</f>
-        <v>0.42,
-[0.4,0.5]</v>
-      </c>
-      <c r="G58" s="14" t="str">
-        <f>G9</f>
-        <v>guyton2006medical,
-valtin1995renal</v>
-      </c>
-      <c r="H58" s="4"/>
-      <c r="I58" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
+        <v>58</v>
+      </c>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8" t="str">
+        <f>F7</f>
+        <v>7.2,
+ [7.35,7.4]</v>
+      </c>
+      <c r="G58" s="8" t="str">
+        <f>G7</f>
+        <v>valentin2002icrp,  guyton2006medical</v>
+      </c>
+      <c r="H58" s="8" t="str">
+        <f>H7</f>
+        <v>p137                                 p384</v>
+      </c>
+      <c r="I58" s="8" t="str">
+        <f>I7</f>
+        <v>Y</v>
+      </c>
+      <c r="J58" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="K58" s="4" t="s">
+        <v>1189</v>
+      </c>
       <c r="L58" s="4"/>
       <c r="M58" s="5" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N58" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O58" s="5" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="P58" s="14"/>
       <c r="Q58" s="14"/>
     </row>
     <row r="59" spans="1:17">
       <c r="A59" s="40" t="s">
-        <v>222</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="E59" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="F59" s="14" t="str">
-        <f>IF(Patient!C2="Male",D59,E59)</f>
-        <v>[13.8,17.2]</v>
-      </c>
-      <c r="G59" s="14" t="str">
-        <f>G34</f>
-        <v>guyton2006medical</v>
-      </c>
-      <c r="H59" s="4"/>
-      <c r="I59" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J59" s="4"/>
+        <v>215</v>
+      </c>
+      <c r="B59" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="G59" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="H59" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J59" s="4" t="s">
+        <v>217</v>
+      </c>
       <c r="K59" s="4"/>
       <c r="L59" s="4"/>
       <c r="M59" s="5" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N59" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O59" s="5" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="P59" s="14"/>
       <c r="Q59" s="14"/>
     </row>
     <row r="60" spans="1:17">
       <c r="A60" s="40" t="s">
-        <v>223</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="14" t="s">
-        <v>225</v>
+        <v>218</v>
+      </c>
+      <c r="B60" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+      <c r="F60" s="8">
+        <v>95</v>
       </c>
       <c r="G60" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="H60" s="5"/>
-      <c r="I60" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J60" s="4"/>
-      <c r="K60" s="41" t="s">
-        <v>227</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="H60" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="I60" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J60" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="K60" s="4"/>
       <c r="L60" s="4"/>
       <c r="M60" s="5" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N60" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O60" s="5" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="P60" s="14"/>
       <c r="Q60" s="14"/>
     </row>
     <row r="61" spans="1:17">
       <c r="A61" s="40" t="s">
-        <v>228</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D61" s="5"/>
-      <c r="E61" s="5"/>
-      <c r="F61" s="14" t="s">
-        <v>229</v>
+        <v>219</v>
+      </c>
+      <c r="B61" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D61" s="8"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="8">
+        <v>40</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="H61" s="4"/>
-      <c r="I61" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J61" s="4"/>
+        <v>15</v>
+      </c>
+      <c r="H61" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="I61" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J61" s="4" t="s">
+        <v>213</v>
+      </c>
       <c r="K61" s="4"/>
       <c r="L61" s="4"/>
       <c r="M61" s="5" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N61" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O61" s="5" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="P61" s="14"/>
       <c r="Q61" s="14"/>
     </row>
-    <row r="62" spans="1:17">
+    <row r="62" spans="1:17" ht="24">
       <c r="A62" s="40" t="s">
-        <v>231</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="42">
-        <v>8.9999999999999999E-8</v>
+        <v>85</v>
+      </c>
+      <c r="B62" s="8"/>
+      <c r="C62" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D62" s="8"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="G62" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="H62" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="I62" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J62" s="4"/>
+        <v>78</v>
+      </c>
+      <c r="H62" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="I62" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>213</v>
+      </c>
       <c r="K62" s="4"/>
       <c r="L62" s="4"/>
       <c r="M62" s="5" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="N62" s="5" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="O62" s="5" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="P62" s="14"/>
       <c r="Q62" s="14"/>
     </row>
-    <row r="63" spans="1:17">
-      <c r="A63" s="40" t="s">
-        <v>234</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="G63" s="43" t="s">
-        <v>236</v>
-      </c>
-      <c r="H63" s="4"/>
-      <c r="I63" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="L63" s="4"/>
-      <c r="M63" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="N63" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="O63" s="5" t="s">
-        <v>1186</v>
-      </c>
-      <c r="P63" s="14"/>
-      <c r="Q63" s="14"/>
+    <row r="63" spans="1:17" ht="24">
+      <c r="A63" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D63" s="9"/>
+      <c r="E63" s="9"/>
+      <c r="F63" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="H63" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I63" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="J63" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="K63" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="L63" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M63" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N63" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="O63" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P63" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q63" s="9" t="s">
+        <v>1194</v>
+      </c>
     </row>
     <row r="64" spans="1:17">
       <c r="A64" s="40" t="s">
-        <v>98</v>
-      </c>
-      <c r="B64" s="14" t="str">
-        <f>B17</f>
-        <v>ct/uL</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="B64" s="4"/>
       <c r="C64" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D64" s="5"/>
       <c r="E64" s="5"/>
-      <c r="F64" s="14">
-        <f>F17</f>
-        <v>5172413.793103449</v>
+      <c r="F64" s="14" t="str">
+        <f>F12</f>
+        <v>0.42,
+[0.4,0.5]</v>
       </c>
       <c r="G64" s="14" t="str">
-        <f>G17</f>
-        <v>guyton2006medical</v>
+        <f>G12</f>
+        <v>guyton2006medical,
+valtin1995renal</v>
       </c>
       <c r="H64" s="4"/>
       <c r="I64" s="5" t="s">
@@ -15903,7 +15942,7 @@
         <v>221</v>
       </c>
       <c r="N64" s="5" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="O64" s="5" t="s">
         <v>1186</v>
@@ -15913,24 +15952,27 @@
     </row>
     <row r="65" spans="1:17">
       <c r="A65" s="40" t="s">
-        <v>118</v>
-      </c>
-      <c r="B65" s="44" t="str">
-        <f>B23</f>
-        <v>ct/uL</v>
+        <v>222</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="C65" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
-      <c r="F65" s="44">
-        <f>F23</f>
-        <v>7000</v>
-      </c>
-      <c r="G65" s="44" t="str">
-        <f>G23</f>
-        <v xml:space="preserve">guyton2006medical   </v>
+      <c r="D65" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="F65" s="14" t="str">
+        <f>IF(Patient!C2="Male",D65,E65)</f>
+        <v>[13.8,17.2]</v>
+      </c>
+      <c r="G65" s="14" t="str">
+        <f>G40</f>
+        <v>guyton2006medical</v>
       </c>
       <c r="H65" s="4"/>
       <c r="I65" s="5" t="s">
@@ -15951,62 +15993,48 @@
       <c r="P65" s="14"/>
       <c r="Q65" s="14"/>
     </row>
-    <row r="66" spans="1:17" ht="24">
-      <c r="A66" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="B66" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="C66" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D66" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="E66" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="F66" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G66" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="H66" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="I66" s="29" t="s">
-        <v>36</v>
-      </c>
-      <c r="J66" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="K66" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="L66" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="M66" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="N66" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="O66" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="P66" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q66" s="9" t="s">
-        <v>1194</v>
-      </c>
+    <row r="66" spans="1:17">
+      <c r="A66" s="40" t="s">
+        <v>223</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="H66" s="5"/>
+      <c r="I66" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J66" s="4"/>
+      <c r="K66" s="41" t="s">
+        <v>227</v>
+      </c>
+      <c r="L66" s="4"/>
+      <c r="M66" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="N66" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O66" s="5" t="s">
+        <v>1186</v>
+      </c>
+      <c r="P66" s="14"/>
+      <c r="Q66" s="14"/>
     </row>
     <row r="67" spans="1:17">
       <c r="A67" s="40" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>110</v>
@@ -16016,13 +16044,11 @@
       </c>
       <c r="D67" s="5"/>
       <c r="E67" s="5"/>
-      <c r="F67" s="14" t="str">
-        <f>F26</f>
-        <v>[4,5]</v>
-      </c>
-      <c r="G67" s="14" t="str">
-        <f>G26</f>
-        <v>valtin1995renal</v>
+      <c r="F67" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>230</v>
       </c>
       <c r="H67" s="4"/>
       <c r="I67" s="5" t="s">
@@ -16032,30 +16058,38 @@
       <c r="K67" s="4"/>
       <c r="L67" s="4"/>
       <c r="M67" s="5" t="s">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="N67" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O67" s="5" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="P67" s="14"/>
       <c r="Q67" s="14"/>
     </row>
     <row r="68" spans="1:17">
       <c r="A68" s="40" t="s">
-        <v>241</v>
-      </c>
-      <c r="B68" s="4"/>
+        <v>231</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>232</v>
+      </c>
       <c r="C68" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D68" s="5"/>
       <c r="E68" s="5"/>
-      <c r="F68" s="14"/>
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
+      <c r="F68" s="42">
+        <v>8.9999999999999999E-8</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" s="5" t="s">
+        <v>233</v>
+      </c>
       <c r="I68" s="5" t="s">
         <v>49</v>
       </c>
@@ -16063,60 +16097,77 @@
       <c r="K68" s="4"/>
       <c r="L68" s="4"/>
       <c r="M68" s="5" t="s">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="N68" s="5" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="O68" s="5" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="P68" s="14"/>
       <c r="Q68" s="14"/>
     </row>
     <row r="69" spans="1:17">
       <c r="A69" s="40" t="s">
-        <v>242</v>
-      </c>
-      <c r="B69" s="4"/>
+        <v>234</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="C69" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D69" s="5"/>
       <c r="E69" s="5"/>
-      <c r="F69" s="14"/>
-      <c r="G69" s="4"/>
+      <c r="F69" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="G69" s="43" t="s">
+        <v>236</v>
+      </c>
       <c r="H69" s="4"/>
       <c r="I69" s="5" t="s">
         <v>49</v>
       </c>
       <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
+      <c r="K69" s="4" t="s">
+        <v>237</v>
+      </c>
       <c r="L69" s="4"/>
       <c r="M69" s="5" t="s">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="N69" s="5" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="O69" s="5" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="P69" s="14"/>
       <c r="Q69" s="14"/>
     </row>
     <row r="70" spans="1:17">
       <c r="A70" s="40" t="s">
-        <v>243</v>
-      </c>
-      <c r="B70" s="4"/>
+        <v>98</v>
+      </c>
+      <c r="B70" s="14" t="str">
+        <f>B23</f>
+        <v>ct/uL</v>
+      </c>
       <c r="C70" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D70" s="5"/>
       <c r="E70" s="5"/>
-      <c r="F70" s="14"/>
-      <c r="G70" s="4"/>
+      <c r="F70" s="14">
+        <f>F23</f>
+        <v>5172413.793103449</v>
+      </c>
+      <c r="G70" s="14" t="str">
+        <f>G23</f>
+        <v>guyton2006medical</v>
+      </c>
       <c r="H70" s="4"/>
       <c r="I70" s="5" t="s">
         <v>49</v>
@@ -16125,38 +16176,37 @@
       <c r="K70" s="4"/>
       <c r="L70" s="4"/>
       <c r="M70" s="5" t="s">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="N70" s="5" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="O70" s="5" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="P70" s="14"/>
       <c r="Q70" s="14"/>
     </row>
     <row r="71" spans="1:17">
       <c r="A71" s="40" t="s">
-        <v>244</v>
-      </c>
-      <c r="B71" s="5" t="s">
-        <v>66</v>
+        <v>118</v>
+      </c>
+      <c r="B71" s="44" t="str">
+        <f>B29</f>
+        <v>ct/uL</v>
       </c>
       <c r="C71" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
-      <c r="F71" s="14" t="str">
-        <f>F6</f>
-        <v>[9.0,18.0],
-[6.0,20.0]</v>
-      </c>
-      <c r="G71" s="14" t="str">
-        <f>G6</f>
-        <v>valtin1995renal,
-Deepakfirst</v>
+      <c r="F71" s="44">
+        <f>F29</f>
+        <v>7000</v>
+      </c>
+      <c r="G71" s="44" t="str">
+        <f>G29</f>
+        <v xml:space="preserve">guyton2006medical   </v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="5" t="s">
@@ -16166,68 +16216,90 @@
       <c r="K71" s="4"/>
       <c r="L71" s="4"/>
       <c r="M71" s="5" t="s">
-        <v>240</v>
+        <v>221</v>
       </c>
       <c r="N71" s="5" t="s">
         <v>71</v>
       </c>
       <c r="O71" s="5" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="P71" s="14"/>
       <c r="Q71" s="14"/>
     </row>
-    <row r="72" spans="1:17">
-      <c r="A72" s="40" t="s">
-        <v>245</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D72" s="5"/>
-      <c r="E72" s="5"/>
-      <c r="F72" s="14" t="str">
-        <f>F28</f>
-        <v>[44.08,52.1]</v>
-      </c>
-      <c r="G72" s="14" t="str">
-        <f>G28</f>
-        <v>cheuvront2014comparison</v>
-      </c>
-      <c r="H72" s="4"/>
-      <c r="I72" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="J72" s="4"/>
-      <c r="K72" s="4"/>
-      <c r="L72" s="4"/>
-      <c r="M72" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="N72" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="O72" s="5" t="s">
-        <v>1187</v>
-      </c>
-      <c r="P72" s="14"/>
-      <c r="Q72" s="14"/>
+    <row r="72" spans="1:17" ht="24">
+      <c r="A72" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E72" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F72" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G72" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="H72" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I72" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="J72" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="K72" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="L72" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M72" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="N72" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="O72" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P72" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q72" s="9" t="s">
+        <v>1194</v>
+      </c>
     </row>
     <row r="73" spans="1:17">
       <c r="A73" s="40" t="s">
-        <v>246</v>
-      </c>
-      <c r="B73" s="14"/>
+        <v>239</v>
+      </c>
+      <c r="B73" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="C73" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
-      <c r="F73" s="14"/>
-      <c r="G73" s="4"/>
+      <c r="F73" s="14" t="str">
+        <f>F32</f>
+        <v>[4,5]</v>
+      </c>
+      <c r="G73" s="14" t="str">
+        <f>G32</f>
+        <v>valtin1995renal</v>
+      </c>
       <c r="H73" s="4"/>
       <c r="I73" s="5" t="s">
         <v>49</v>
@@ -16249,23 +16321,16 @@
     </row>
     <row r="74" spans="1:17">
       <c r="A74" s="40" t="s">
-        <v>247</v>
-      </c>
-      <c r="B74" s="14" t="s">
-        <v>89</v>
-      </c>
+        <v>241</v>
+      </c>
+      <c r="B74" s="4"/>
       <c r="C74" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
-      <c r="F74" s="14" t="s">
-        <v>248</v>
-      </c>
-      <c r="G74" s="14" t="str">
-        <f>G27</f>
-        <v>valtin1995renal</v>
-      </c>
+      <c r="F74" s="14"/>
+      <c r="G74" s="4"/>
       <c r="H74" s="4"/>
       <c r="I74" s="5" t="s">
         <v>49</v>
@@ -16287,24 +16352,16 @@
     </row>
     <row r="75" spans="1:17">
       <c r="A75" s="40" t="s">
-        <v>249</v>
-      </c>
-      <c r="B75" s="5" t="s">
-        <v>128</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="B75" s="4"/>
       <c r="C75" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
-      <c r="F75" s="14" t="str">
-        <f>F30</f>
-        <v>[5.0,15.0]</v>
-      </c>
-      <c r="G75" s="14" t="str">
-        <f>G30</f>
-        <v>valtin1995renal</v>
-      </c>
+      <c r="F75" s="14"/>
+      <c r="G75" s="4"/>
       <c r="H75" s="4"/>
       <c r="I75" s="5" t="s">
         <v>49</v>
@@ -16326,22 +16383,16 @@
     </row>
     <row r="76" spans="1:17">
       <c r="A76" s="40" t="s">
-        <v>250</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>66</v>
-      </c>
+        <v>243</v>
+      </c>
+      <c r="B76" s="4"/>
       <c r="C76" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
-      <c r="F76" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="G76" s="14" t="s">
-        <v>91</v>
-      </c>
+      <c r="F76" s="14"/>
+      <c r="G76" s="4"/>
       <c r="H76" s="4"/>
       <c r="I76" s="5" t="s">
         <v>49</v>
@@ -16363,16 +16414,26 @@
     </row>
     <row r="77" spans="1:17">
       <c r="A77" s="40" t="s">
-        <v>252</v>
-      </c>
-      <c r="B77" s="4"/>
+        <v>244</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>66</v>
+      </c>
       <c r="C77" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D77" s="5"/>
       <c r="E77" s="5"/>
-      <c r="F77" s="14"/>
-      <c r="G77" s="4"/>
+      <c r="F77" s="14" t="str">
+        <f>F9</f>
+        <v>[9.0,18.0],
+[6.0,20.0]</v>
+      </c>
+      <c r="G77" s="14" t="str">
+        <f>G9</f>
+        <v>valtin1995renal,
+Deepakfirst</v>
+      </c>
       <c r="H77" s="4"/>
       <c r="I77" s="5" t="s">
         <v>49</v>
@@ -16394,23 +16455,23 @@
     </row>
     <row r="78" spans="1:17">
       <c r="A78" s="40" t="s">
-        <v>253</v>
-      </c>
-      <c r="B78" s="18" t="s">
-        <v>89</v>
+        <v>245</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>128</v>
       </c>
       <c r="C78" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D78" s="5"/>
       <c r="E78" s="5"/>
-      <c r="F78" s="14" t="s">
-        <v>254</v>
+      <c r="F78" s="14" t="str">
+        <f>F34</f>
+        <v>[44.08,52.1]</v>
       </c>
       <c r="G78" s="14" t="str">
-        <f>G38</f>
-        <v>Leeuwen2015laboratory,
-valtin1995renal</v>
+        <f>G34</f>
+        <v>cheuvront2014comparison</v>
       </c>
       <c r="H78" s="4"/>
       <c r="I78" s="5" t="s">
@@ -16433,9 +16494,9 @@
     </row>
     <row r="79" spans="1:17">
       <c r="A79" s="40" t="s">
-        <v>255</v>
-      </c>
-      <c r="B79" s="4"/>
+        <v>246</v>
+      </c>
+      <c r="B79" s="14"/>
       <c r="C79" s="5" t="s">
         <v>46</v>
       </c>
@@ -16464,29 +16525,28 @@
     </row>
     <row r="80" spans="1:17">
       <c r="A80" s="40" t="s">
-        <v>256</v>
-      </c>
-      <c r="B80" s="18" t="s">
-        <v>110</v>
+        <v>247</v>
+      </c>
+      <c r="B80" s="14" t="s">
+        <v>89</v>
       </c>
       <c r="C80" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D80" s="5"/>
       <c r="E80" s="5"/>
-      <c r="F80" s="14" t="str">
-        <f>F20</f>
-        <v>[6,8]</v>
+      <c r="F80" s="14" t="s">
+        <v>248</v>
       </c>
       <c r="G80" s="14" t="str">
-        <f>G20</f>
+        <f>G33</f>
         <v>valtin1995renal</v>
       </c>
       <c r="H80" s="4"/>
       <c r="I80" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="J80" s="14"/>
+      <c r="J80" s="4"/>
       <c r="K80" s="4"/>
       <c r="L80" s="4"/>
       <c r="M80" s="5" t="s">
@@ -16501,24 +16561,240 @@
       <c r="P80" s="14"/>
       <c r="Q80" s="14"/>
     </row>
-    <row r="81" spans="15:15">
-      <c r="O81" s="45"/>
+    <row r="81" spans="1:17">
+      <c r="A81" s="40" t="s">
+        <v>249</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C81" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D81" s="5"/>
+      <c r="E81" s="5"/>
+      <c r="F81" s="14" t="str">
+        <f>F36</f>
+        <v>[5.0,15.0]</v>
+      </c>
+      <c r="G81" s="14" t="str">
+        <f>G36</f>
+        <v>valtin1995renal</v>
+      </c>
+      <c r="H81" s="4"/>
+      <c r="I81" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J81" s="4"/>
+      <c r="K81" s="4"/>
+      <c r="L81" s="4"/>
+      <c r="M81" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="N81" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O81" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="P81" s="14"/>
+      <c r="Q81" s="14"/>
+    </row>
+    <row r="82" spans="1:17">
+      <c r="A82" s="40" t="s">
+        <v>250</v>
+      </c>
+      <c r="B82" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D82" s="5"/>
+      <c r="E82" s="5"/>
+      <c r="F82" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="G82" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="H82" s="4"/>
+      <c r="I82" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J82" s="4"/>
+      <c r="K82" s="4"/>
+      <c r="L82" s="4"/>
+      <c r="M82" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="N82" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O82" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="P82" s="14"/>
+      <c r="Q82" s="14"/>
+    </row>
+    <row r="83" spans="1:17">
+      <c r="A83" s="40" t="s">
+        <v>252</v>
+      </c>
+      <c r="B83" s="4"/>
+      <c r="C83" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D83" s="5"/>
+      <c r="E83" s="5"/>
+      <c r="F83" s="14"/>
+      <c r="G83" s="4"/>
+      <c r="H83" s="4"/>
+      <c r="I83" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J83" s="4"/>
+      <c r="K83" s="4"/>
+      <c r="L83" s="4"/>
+      <c r="M83" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="N83" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O83" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="P83" s="14"/>
+      <c r="Q83" s="14"/>
+    </row>
+    <row r="84" spans="1:17">
+      <c r="A84" s="40" t="s">
+        <v>253</v>
+      </c>
+      <c r="B84" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D84" s="5"/>
+      <c r="E84" s="5"/>
+      <c r="F84" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="G84" s="14" t="str">
+        <f>G44</f>
+        <v>Leeuwen2015laboratory,
+valtin1995renal</v>
+      </c>
+      <c r="H84" s="4"/>
+      <c r="I84" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J84" s="4"/>
+      <c r="K84" s="4"/>
+      <c r="L84" s="4"/>
+      <c r="M84" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="N84" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O84" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="P84" s="14"/>
+      <c r="Q84" s="14"/>
+    </row>
+    <row r="85" spans="1:17">
+      <c r="A85" s="40" t="s">
+        <v>255</v>
+      </c>
+      <c r="B85" s="4"/>
+      <c r="C85" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D85" s="5"/>
+      <c r="E85" s="5"/>
+      <c r="F85" s="14"/>
+      <c r="G85" s="4"/>
+      <c r="H85" s="4"/>
+      <c r="I85" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J85" s="4"/>
+      <c r="K85" s="4"/>
+      <c r="L85" s="4"/>
+      <c r="M85" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="N85" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O85" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="P85" s="14"/>
+      <c r="Q85" s="14"/>
+    </row>
+    <row r="86" spans="1:17">
+      <c r="A86" s="40" t="s">
+        <v>256</v>
+      </c>
+      <c r="B86" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D86" s="5"/>
+      <c r="E86" s="5"/>
+      <c r="F86" s="14" t="str">
+        <f>F26</f>
+        <v>[6,8]</v>
+      </c>
+      <c r="G86" s="14" t="str">
+        <f>G26</f>
+        <v>valtin1995renal</v>
+      </c>
+      <c r="H86" s="4"/>
+      <c r="I86" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J86" s="14"/>
+      <c r="K86" s="4"/>
+      <c r="L86" s="4"/>
+      <c r="M86" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="N86" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O86" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="P86" s="14"/>
+      <c r="Q86" s="14"/>
+    </row>
+    <row r="87" spans="1:17">
+      <c r="O87" s="45"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="L13" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="L34" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="L41" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="K60" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
-    <hyperlink ref="O52" r:id="rId5" xr:uid="{77CFD383-FFBB-43C3-9719-6C8925AAAF78}"/>
-    <hyperlink ref="O53" r:id="rId6" xr:uid="{FC8D543E-EB3E-4309-9928-49CA2DE8AE52}"/>
-    <hyperlink ref="O54" r:id="rId7" xr:uid="{DBD15686-F216-4EDA-9421-9DE799BC92F4}"/>
-    <hyperlink ref="O55" r:id="rId8" xr:uid="{8D9A9D3D-AD62-4201-ACA3-FDDCAEB5E9FC}"/>
-    <hyperlink ref="O56" r:id="rId9" xr:uid="{0042DED4-84E3-45EF-B81A-33C49E246FFA}"/>
-    <hyperlink ref="O58" r:id="rId10" xr:uid="{20112368-58A2-4555-8B18-514CF165C0FC}"/>
-    <hyperlink ref="O59:O65" r:id="rId11" display="CBC@120s" xr:uid="{20D8E90A-E850-443A-BB57-0CD158AC0414}"/>
-    <hyperlink ref="O67" r:id="rId12" xr:uid="{0318CE1E-6F08-4524-A904-03D995DB5DB1}"/>
-    <hyperlink ref="O68:O80" r:id="rId13" display="CMP@120s" xr:uid="{C869CBFA-5948-401B-822D-A99AAEA40075}"/>
+    <hyperlink ref="L19" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="L40" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="L47" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="K66" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="O58" r:id="rId5" xr:uid="{77CFD383-FFBB-43C3-9719-6C8925AAAF78}"/>
+    <hyperlink ref="O59" r:id="rId6" xr:uid="{FC8D543E-EB3E-4309-9928-49CA2DE8AE52}"/>
+    <hyperlink ref="O60" r:id="rId7" xr:uid="{DBD15686-F216-4EDA-9421-9DE799BC92F4}"/>
+    <hyperlink ref="O61" r:id="rId8" xr:uid="{8D9A9D3D-AD62-4201-ACA3-FDDCAEB5E9FC}"/>
+    <hyperlink ref="O62" r:id="rId9" xr:uid="{0042DED4-84E3-45EF-B81A-33C49E246FFA}"/>
+    <hyperlink ref="O64" r:id="rId10" xr:uid="{20112368-58A2-4555-8B18-514CF165C0FC}"/>
+    <hyperlink ref="O65:O71" r:id="rId11" display="CBC@120s" xr:uid="{20D8E90A-E850-443A-BB57-0CD158AC0414}"/>
+    <hyperlink ref="O73" r:id="rId12" xr:uid="{0318CE1E-6F08-4524-A904-03D995DB5DB1}"/>
+    <hyperlink ref="O74:O86" r:id="rId13" display="CMP@120s" xr:uid="{C869CBFA-5948-401B-822D-A99AAEA40075}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Fix system data validation spreadsheet typo.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/SystemValidationData.xlsx
+++ b/data/human/adult/validation/SystemValidationData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94AC0127-FEB7-48AF-AE43-6E91CF4DACFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0EF5D0-CF4A-4CA9-BCE4-CBF453498BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18765" yWindow="4260" windowWidth="34530" windowHeight="26775" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18420" yWindow="3915" windowWidth="34530" windowHeight="26775" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient" sheetId="1" r:id="rId1"/>
@@ -3792,13 +3792,13 @@
     <t>[0.18,0.20]</t>
   </si>
   <si>
-    <t>[0.04-0.05]</t>
-  </si>
-  <si>
     <t>[0.13,0.15]</t>
   </si>
   <si>
     <t>ClinicalOxygenConsumption</t>
+  </si>
+  <si>
+    <t>[0.04,0.05]</t>
   </si>
 </sst>
 </file>
@@ -13431,7 +13431,7 @@
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8" t="s">
-        <v>1206</v>
+        <v>1208</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>15</v>
@@ -13730,7 +13730,7 @@
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="10" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>14</v>
@@ -13860,7 +13860,7 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="8" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Support validation of the expanded lungs engine configuration
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/SystemValidationData.xlsx
+++ b/data/human/adult/validation/SystemValidationData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAEE00C0-82DE-41C1-8440-323DE0D8DAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45ECEB53-8FFA-45EC-BFAC-0D7B86DA64C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Patient" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,6 @@
     <sheet name="RespiratoryExpandedLungs" sheetId="12" r:id="rId12"/>
     <sheet name="Tissue" sheetId="11" r:id="rId13"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId14"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -48,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7003" uniqueCount="1250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7005" uniqueCount="1250">
   <si>
     <t>Patient Inputs</t>
   </si>
@@ -4632,52 +4629,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Patient"/>
-      <sheetName val="Blood Chemistry"/>
-      <sheetName val="Cardiovascular"/>
-      <sheetName val="CardiovascularExpandedLungs"/>
-      <sheetName val="CardiovascularComputationalLife"/>
-      <sheetName val="Endocrine"/>
-      <sheetName val="Energy"/>
-      <sheetName val="Gastrointestinal"/>
-      <sheetName val="Nervous"/>
-      <sheetName val="Renal"/>
-      <sheetName val="Respiratory"/>
-      <sheetName val="RespiratoryExpandedLungs"/>
-      <sheetName val="Tissue"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10">
-        <row r="55">
-          <cell r="F55">
-            <v>8.4000000000000005E-2</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
@@ -16004,7 +15955,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1552AE4F-8EDA-4B53-A93F-ABC6B36E30F3}">
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.42578125" customWidth="1"/>
@@ -16022,7 +15973,7 @@
     <col min="15" max="15" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="24">
+    <row r="1" spans="1:17" ht="24">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -16071,8 +16022,11 @@
       <c r="P1" s="9" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:16">
+      <c r="Q1" s="9" t="s">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="67" t="s">
         <v>1230</v>
       </c>
@@ -16085,7 +16039,7 @@
       <c r="D2" s="20"/>
       <c r="E2" s="20"/>
       <c r="F2" s="122">
-        <f>(K2/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K2/100*Respiratory!$F$56)*1000</f>
         <v>3.3801600000000001</v>
       </c>
       <c r="G2" s="51" t="s">
@@ -16112,8 +16066,9 @@
       <c r="P2" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:16">
+      <c r="Q2" s="14"/>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="67" t="s">
         <v>1229</v>
       </c>
@@ -16126,7 +16081,7 @@
       <c r="D3" s="20"/>
       <c r="E3" s="20"/>
       <c r="F3" s="122">
-        <f>(K3/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K3/100*Respiratory!$F$56)*1000</f>
         <v>3.7111200000000006</v>
       </c>
       <c r="G3" s="51" t="s">
@@ -16153,8 +16108,9 @@
       <c r="P3" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:16">
+      <c r="Q3" s="14"/>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="67" t="s">
         <v>1228</v>
       </c>
@@ -16167,7 +16123,7 @@
       <c r="D4" s="20"/>
       <c r="E4" s="20"/>
       <c r="F4" s="122">
-        <f>(K4/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K4/100*Respiratory!$F$56)*1000</f>
         <v>4.1806799999999997</v>
       </c>
       <c r="G4" s="51" t="s">
@@ -16194,8 +16150,9 @@
       <c r="P4" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:16">
+      <c r="Q4" s="14"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="67" t="s">
         <v>1227</v>
       </c>
@@ -16208,7 +16165,7 @@
       <c r="D5" s="20"/>
       <c r="E5" s="20"/>
       <c r="F5" s="122">
-        <f>(K5/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K5/100*Respiratory!$F$56)*1000</f>
         <v>4.9534800000000008</v>
       </c>
       <c r="G5" s="51" t="s">
@@ -16235,8 +16192,9 @@
       <c r="P5" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="Q5" s="14"/>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="67" t="s">
         <v>1226</v>
       </c>
@@ -16249,7 +16207,7 @@
       <c r="D6" s="20"/>
       <c r="E6" s="20"/>
       <c r="F6" s="122">
-        <f>(K6/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K6/100*Respiratory!$F$56)*1000</f>
         <v>4.8980399999999999</v>
       </c>
       <c r="G6" s="51" t="s">
@@ -16276,8 +16234,9 @@
       <c r="P6" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="Q6" s="14"/>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="67" t="s">
         <v>1225</v>
       </c>
@@ -16290,7 +16249,7 @@
       <c r="D7" s="20"/>
       <c r="E7" s="20"/>
       <c r="F7" s="122">
-        <f>(K7/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K7/100*Respiratory!$F$56)*1000</f>
         <v>4.4293200000000006</v>
       </c>
       <c r="G7" s="51" t="s">
@@ -16317,8 +16276,9 @@
       <c r="P7" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="Q7" s="14"/>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="67" t="s">
         <v>1224</v>
       </c>
@@ -16331,7 +16291,7 @@
       <c r="D8" s="20"/>
       <c r="E8" s="20"/>
       <c r="F8" s="122">
-        <f>(K8/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K8/100*Respiratory!$F$56)*1000</f>
         <v>5.0635200000000005</v>
       </c>
       <c r="G8" s="51" t="s">
@@ -16358,8 +16318,9 @@
       <c r="P8" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:16">
+      <c r="Q8" s="14"/>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" s="67" t="s">
         <v>1223</v>
       </c>
@@ -16372,7 +16333,7 @@
       <c r="D9" s="20"/>
       <c r="E9" s="20"/>
       <c r="F9" s="122">
-        <f>(K9/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K9/100*Respiratory!$F$56)*1000</f>
         <v>5.3121600000000004</v>
       </c>
       <c r="G9" s="51" t="s">
@@ -16399,8 +16360,9 @@
       <c r="P9" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="Q9" s="14"/>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10" s="67" t="s">
         <v>1222</v>
       </c>
@@ -16413,7 +16375,7 @@
       <c r="D10" s="20"/>
       <c r="E10" s="20"/>
       <c r="F10" s="122">
-        <f>(K10/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K10/100*Respiratory!$F$56)*1000</f>
         <v>5.4230400000000003</v>
       </c>
       <c r="G10" s="51" t="s">
@@ -16440,8 +16402,9 @@
       <c r="P10" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="Q10" s="14"/>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11" s="67" t="s">
         <v>1221</v>
       </c>
@@ -16454,7 +16417,7 @@
       <c r="D11" s="20"/>
       <c r="E11" s="20"/>
       <c r="F11" s="122">
-        <f>(K11/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K11/100*Respiratory!$F$56)*1000</f>
         <v>5.1744000000000012</v>
       </c>
       <c r="G11" s="51" t="s">
@@ -16481,8 +16444,9 @@
       <c r="P11" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="Q11" s="14"/>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12" s="67" t="s">
         <v>1220</v>
       </c>
@@ -16495,7 +16459,7 @@
       <c r="D12" s="20"/>
       <c r="E12" s="20"/>
       <c r="F12" s="122">
-        <f>(K12/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K12/100*Respiratory!$F$56)*1000</f>
         <v>5.2021199999999999</v>
       </c>
       <c r="G12" s="51" t="s">
@@ -16522,8 +16486,9 @@
       <c r="P12" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="Q12" s="14"/>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13" s="67" t="s">
         <v>1219</v>
       </c>
@@ -16536,7 +16501,7 @@
       <c r="D13" s="20"/>
       <c r="E13" s="20"/>
       <c r="F13" s="122">
-        <f>(K13/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K13/100*Respiratory!$F$56)*1000</f>
         <v>5.3676000000000004</v>
       </c>
       <c r="G13" s="51" t="s">
@@ -16563,8 +16528,9 @@
       <c r="P13" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:16">
+      <c r="Q13" s="14"/>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" s="67" t="s">
         <v>1218</v>
       </c>
@@ -16577,7 +16543,7 @@
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
       <c r="F14" s="122">
-        <f>(K14/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K14/100*Respiratory!$F$56)*1000</f>
         <v>5.1189600000000004</v>
       </c>
       <c r="G14" s="51" t="s">
@@ -16604,8 +16570,9 @@
       <c r="P14" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="Q14" s="14"/>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" s="67" t="s">
         <v>1217</v>
       </c>
@@ -16618,7 +16585,7 @@
       <c r="D15" s="20"/>
       <c r="E15" s="20"/>
       <c r="F15" s="122">
-        <f>(K15/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K15/100*Respiratory!$F$56)*1000</f>
         <v>4.4293200000000006</v>
       </c>
       <c r="G15" s="51" t="s">
@@ -16645,8 +16612,9 @@
       <c r="P15" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="Q15" s="14"/>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="67" t="s">
         <v>1216</v>
       </c>
@@ -16659,7 +16627,7 @@
       <c r="D16" s="20"/>
       <c r="E16" s="20"/>
       <c r="F16" s="122">
-        <f>(K16/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K16/100*Respiratory!$F$56)*1000</f>
         <v>5.0089200000000007</v>
       </c>
       <c r="G16" s="51" t="s">
@@ -16686,8 +16654,9 @@
       <c r="P16" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:16">
+      <c r="Q16" s="14"/>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" s="67" t="s">
         <v>1215</v>
       </c>
@@ -16700,7 +16669,7 @@
       <c r="D17" s="20"/>
       <c r="E17" s="20"/>
       <c r="F17" s="122">
-        <f>(K17/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K17/100*Respiratory!$F$56)*1000</f>
         <v>4.6771199999999995</v>
       </c>
       <c r="G17" s="51" t="s">
@@ -16727,8 +16696,9 @@
       <c r="P17" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="18" spans="1:16">
+      <c r="Q17" s="14"/>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" s="67" t="s">
         <v>1214</v>
       </c>
@@ -16741,7 +16711,7 @@
       <c r="D18" s="20"/>
       <c r="E18" s="20"/>
       <c r="F18" s="122">
-        <f>(K18/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K18/100*Respiratory!$F$56)*1000</f>
         <v>4.1252399999999998</v>
       </c>
       <c r="G18" s="51" t="s">
@@ -16768,8 +16738,9 @@
       <c r="P18" s="66">
         <v>4</v>
       </c>
-    </row>
-    <row r="19" spans="1:16">
+      <c r="Q18" s="14"/>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="67" t="s">
         <v>1213</v>
       </c>
@@ -16782,7 +16753,7 @@
       <c r="D19" s="20"/>
       <c r="E19" s="20"/>
       <c r="F19" s="122">
-        <f>(K19/100*[1]Respiratory!$F$55)*1000</f>
+        <f>(K19/100*Respiratory!$F$56)*1000</f>
         <v>3.5456400000000001</v>
       </c>
       <c r="G19" s="51" t="s">
@@ -16809,6 +16780,7 @@
       <c r="P19" s="66">
         <v>4</v>
       </c>
+      <c r="Q19" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -28928,7 +28900,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16A288E4-2A5B-49C3-8F74-67B83EE55504}">
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="65.5703125" customWidth="1"/>
@@ -28946,7 +28918,7 @@
     <col min="15" max="15" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="24">
+    <row r="1" spans="1:17" ht="24">
       <c r="A1" s="3" t="s">
         <v>30</v>
       </c>
@@ -28995,8 +28967,11 @@
       <c r="P1" s="9" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:16">
+      <c r="Q1" s="9" t="s">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2" s="10" t="s">
         <v>1249</v>
       </c>
@@ -29034,8 +29009,9 @@
         <v>356</v>
       </c>
       <c r="P2" s="14"/>
-    </row>
-    <row r="3" spans="1:16">
+      <c r="Q2" s="14"/>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3" s="10" t="s">
         <v>1248</v>
       </c>
@@ -29073,8 +29049,9 @@
         <v>356</v>
       </c>
       <c r="P3" s="14"/>
-    </row>
-    <row r="4" spans="1:16">
+      <c r="Q3" s="14"/>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4" s="10" t="s">
         <v>1247</v>
       </c>
@@ -29112,8 +29089,9 @@
         <v>356</v>
       </c>
       <c r="P4" s="14"/>
-    </row>
-    <row r="5" spans="1:16">
+      <c r="Q4" s="14"/>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5" s="10" t="s">
         <v>1246</v>
       </c>
@@ -29151,8 +29129,9 @@
         <v>356</v>
       </c>
       <c r="P5" s="14"/>
-    </row>
-    <row r="6" spans="1:16">
+      <c r="Q5" s="14"/>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6" s="10" t="s">
         <v>1245</v>
       </c>
@@ -29190,8 +29169,9 @@
         <v>356</v>
       </c>
       <c r="P6" s="14"/>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="Q6" s="14"/>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7" s="10" t="s">
         <v>1244</v>
       </c>
@@ -29229,8 +29209,9 @@
         <v>356</v>
       </c>
       <c r="P7" s="14"/>
-    </row>
-    <row r="8" spans="1:16">
+      <c r="Q7" s="14"/>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8" s="10" t="s">
         <v>1243</v>
       </c>
@@ -29268,8 +29249,9 @@
         <v>356</v>
       </c>
       <c r="P8" s="14"/>
-    </row>
-    <row r="9" spans="1:16">
+      <c r="Q8" s="14"/>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9" s="10" t="s">
         <v>1242</v>
       </c>
@@ -29307,8 +29289,9 @@
         <v>356</v>
       </c>
       <c r="P9" s="14"/>
-    </row>
-    <row r="10" spans="1:16">
+      <c r="Q9" s="14"/>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10" s="10" t="s">
         <v>1241</v>
       </c>
@@ -29346,8 +29329,9 @@
         <v>356</v>
       </c>
       <c r="P10" s="14"/>
-    </row>
-    <row r="11" spans="1:16">
+      <c r="Q10" s="14"/>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11" s="10" t="s">
         <v>1240</v>
       </c>
@@ -29385,8 +29369,9 @@
         <v>356</v>
       </c>
       <c r="P11" s="14"/>
-    </row>
-    <row r="12" spans="1:16">
+      <c r="Q11" s="14"/>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12" s="10" t="s">
         <v>1239</v>
       </c>
@@ -29424,8 +29409,9 @@
         <v>356</v>
       </c>
       <c r="P12" s="14"/>
-    </row>
-    <row r="13" spans="1:16">
+      <c r="Q12" s="14"/>
+    </row>
+    <row r="13" spans="1:17">
       <c r="A13" s="10" t="s">
         <v>1238</v>
       </c>
@@ -29463,8 +29449,9 @@
         <v>356</v>
       </c>
       <c r="P13" s="14"/>
-    </row>
-    <row r="14" spans="1:16">
+      <c r="Q13" s="14"/>
+    </row>
+    <row r="14" spans="1:17">
       <c r="A14" s="10" t="s">
         <v>1237</v>
       </c>
@@ -29502,8 +29489,9 @@
         <v>356</v>
       </c>
       <c r="P14" s="14"/>
-    </row>
-    <row r="15" spans="1:16">
+      <c r="Q14" s="14"/>
+    </row>
+    <row r="15" spans="1:17">
       <c r="A15" s="10" t="s">
         <v>1236</v>
       </c>
@@ -29541,8 +29529,9 @@
         <v>356</v>
       </c>
       <c r="P15" s="14"/>
-    </row>
-    <row r="16" spans="1:16">
+      <c r="Q15" s="14"/>
+    </row>
+    <row r="16" spans="1:17">
       <c r="A16" s="10" t="s">
         <v>1235</v>
       </c>
@@ -29580,8 +29569,9 @@
         <v>356</v>
       </c>
       <c r="P16" s="14"/>
-    </row>
-    <row r="17" spans="1:16">
+      <c r="Q16" s="14"/>
+    </row>
+    <row r="17" spans="1:17">
       <c r="A17" s="10" t="s">
         <v>1234</v>
       </c>
@@ -29619,8 +29609,9 @@
         <v>356</v>
       </c>
       <c r="P17" s="14"/>
-    </row>
-    <row r="18" spans="1:16">
+      <c r="Q17" s="14"/>
+    </row>
+    <row r="18" spans="1:17">
       <c r="A18" s="10" t="s">
         <v>1233</v>
       </c>
@@ -29658,8 +29649,9 @@
         <v>356</v>
       </c>
       <c r="P18" s="14"/>
-    </row>
-    <row r="19" spans="1:16">
+      <c r="Q18" s="14"/>
+    </row>
+    <row r="19" spans="1:17">
       <c r="A19" s="10" t="s">
         <v>1232</v>
       </c>
@@ -29697,6 +29689,7 @@
         <v>356</v>
       </c>
       <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>